<commit_message>
RX 235.58 -> 234.75: 702 Shuttles 10:50 from Primm to Barstow reaches the San Bernardino anchor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/route_legs.xlsx
+++ b/docs/route_legs.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Wheeling 234.24" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Control 237.24" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="RX 235.58" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="RX 234.75" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="MEX 237.75" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="X_TOL 237.91" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="X 238.11" sheetId="6" state="visible" r:id="rId6"/>
@@ -8839,7 +8839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8862,7 +8862,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RX 235.58: 235.58 h, first bus d1 Thu 10:00, finish d11 Sun 06:35</t>
+          <t>RX 234.75: 234.75 h, first bus d1 Thu 10:50, finish d11 Sun 06:35</t>
         </is>
       </c>
     </row>
@@ -8961,12 +8961,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>d1 Thu 10:00</t>
+          <t>d1 Thu 10:50</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Las Vegas Bus Terminal</t>
+          <t>Primm Bus Stop (702 Shuttles)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -8976,12 +8976,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>d1 Thu 14:35</t>
+          <t>d1 Thu 12:27</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>San Bernardino Depot</t>
+          <t>Barstow East Main St 1611 (702 Shuttles)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -8989,17 +8989,17 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Greyhound-us: Los Angeles - Las Vegas</t>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>702 Shuttles: Las Vegas -&gt; Ontario (Nick screenshot Oct 2 2026, Primm 10:50 to Ontario 13:37; Las Vegas and Jean times inferred from the 15:15 run; daily assumed; Ontario stop point approximate)</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>4.58</v>
+        <v>1.62</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
-        <v>3.7</v>
+        <v>5</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -9009,7 +9009,11 @@
       <c r="N4" t="n">
         <v>2</v>
       </c>
-      <c r="O4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -9017,17 +9021,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>d1 Thu 15:10</t>
+          <t>d1 Thu 12:27</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>San Bernardino Depot</t>
+          <t>Barstow East Main St 1611 (702 Shuttles)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -9037,46 +9041,34 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>d2 Fri 21:15</t>
+          <t>d1 Thu 12:40</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Oklahoma City Bus Station</t>
+          <t>Barstow Station</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Greyhound-us: St Louis - Albuquerque - Los Angeles</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>28.08</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>AZ NM OK TX</t>
-        </is>
-      </c>
+        <v>0.22</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>6</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -9089,59 +9081,55 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>d2 Fri 22:40</t>
+          <t>d1 Thu 12:55</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Oklahoma City Bus Station</t>
+          <t>Barstow Station</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>d3 Sat 08:00</t>
+          <t>d1 Thu 14:35</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Memphis Bus Station</t>
+          <t>San Bernardino Depot</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Greyhound-us: Oklahoma City - Memphis</t>
+          <t>Greyhound-us: Los Angeles - Las Vegas</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>9.33</v>
-      </c>
-      <c r="K6" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>AR TN</t>
-        </is>
-      </c>
+        <v>1.67</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L6" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>daily anchor</t>
+          <t>tight</t>
         </is>
       </c>
     </row>
@@ -9156,57 +9144,61 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>d3 Sat 08:50</t>
+          <t>d1 Thu 15:10</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Memphis Bus Station</t>
+          <t>San Bernardino Depot</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>d3 Sat 17:50</t>
+          <t>d2 Fri 21:15</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>New Orleans Bus Station</t>
+          <t>Oklahoma City Bus Station</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Greyhound-us: Baton Rouge - New Orleans - Memphis</t>
+          <t>Greyhound-us: St Louis - Albuquerque - Los Angeles</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>9</v>
+        <v>28.08</v>
       </c>
       <c r="K7" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="L7" t="n">
-        <v>11.9</v>
+        <v>0.58</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>LA MS</t>
+          <t>AZ NM OK TX</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>10</v>
-      </c>
-      <c r="O7" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -9219,55 +9211,59 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>d3 Sat 18:00</t>
+          <t>d2 Fri 22:40</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>New Orleans Bus Station</t>
+          <t>Oklahoma City Bus Station</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>d3 Sat 21:15</t>
+          <t>d3 Sat 08:00</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Lafayette Transit System</t>
+          <t>Memphis Bus Station</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Greyhound-us: Atlanta - New Orleans - Houston</t>
+          <t>Greyhound-us: Oklahoma City - Memphis</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="K8" s="5" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="L8" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
+        <v>9.33</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>AR TN</t>
+        </is>
+      </c>
       <c r="N8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>tight</t>
+          <t>daily anchor</t>
         </is>
       </c>
     </row>
@@ -9282,61 +9278,57 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>d3 Sat 22:35</t>
+          <t>d3 Sat 08:50</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Lafayette Transit System</t>
+          <t>Memphis Bus Station</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>d3 Sat 17:50</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>New Orleans Bus Station</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>LA</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>d4 Sun 11:00</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Greyhound-us: Orlando - Houston</t>
+          <t>Greyhound-us: Baton Rouge - New Orleans - Memphis</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>11.42</v>
+        <v>9</v>
       </c>
       <c r="K9" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="L9" s="4" t="n">
-        <v>24</v>
+        <v>0.83</v>
+      </c>
+      <c r="L9" t="n">
+        <v>11.9</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>AL FL</t>
+          <t>LA MS</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>12</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -9349,53 +9341,57 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>d4 Sun 11:25</t>
+          <t>d3 Sat 18:00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
+          <t>New Orleans Bus Station</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>d4 Sun 14:50</t>
+          <t>d3 Sat 21:15</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Jacksonville (Downtown)</t>
+          <t>Lafayette Transit System</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Greyhound-us: Jacksonville - Mobile</t>
+          <t>Greyhound-us: Atlanta - New Orleans - Houston</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>3.42</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.42</v>
+        <v>3.25</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>0.17</v>
       </c>
       <c r="L10" t="n">
-        <v>5.8</v>
+        <v>11.8</v>
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>12</v>
-      </c>
-      <c r="O10" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -9403,54 +9399,66 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>d4 Sun 14:50</t>
+          <t>d3 Sat 22:35</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Jacksonville (Downtown)</t>
+          <t>Lafayette Transit System</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>d4 Sun 11:00</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>d4 Sun 14:50</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>JRTC Bay H</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Greyhound-us: Orlando - Houston</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+        <v>11.42</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>AL FL</t>
+        </is>
+      </c>
       <c r="N11" t="n">
         <v>12</v>
       </c>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -9463,12 +9471,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>d4 Sun 15:00</t>
+          <t>d4 Sun 11:25</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>JRTC Bay H</t>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -9478,12 +9486,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>d4 Sun 15:27</t>
+          <t>d4 Sun 14:50</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Amtrak Station</t>
+          <t>Jacksonville (Downtown)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -9493,27 +9501,23 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Jacksonville Transportation Authority: Kings Road</t>
+          <t>Greyhound-us: Jacksonville - Mobile</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="K12" s="5" t="n">
-        <v>0.15</v>
+        <v>3.42</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.42</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>5.8</v>
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
         <v>12</v>
       </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>tight</t>
-        </is>
-      </c>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -9526,12 +9530,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>d4 Sun 15:27</t>
+          <t>d4 Sun 14:50</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Amtrak Station</t>
+          <t>Jacksonville (Downtown)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -9541,12 +9545,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>d4 Sun 15:35</t>
+          <t>d4 Sun 14:50</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>JRTC Bay H</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -9560,7 +9564,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0.14</v>
+        <v>0.02</v>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -9581,12 +9585,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>d4 Sun 16:11</t>
+          <t>d4 Sun 15:00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>JRTC Bay H</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -9596,38 +9600,42 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>d5 Mon 06:25</t>
+          <t>d4 Sun 15:27</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>Amtrak Station</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Amtrak: Silver Meteor</t>
+          <t>Jacksonville Transportation Authority: Kings Road</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>14.23</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0.59</v>
+        <v>0.45</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>0.15</v>
       </c>
       <c r="L14" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>GA NC SC VA</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>16</v>
-      </c>
-      <c r="O14" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9635,56 +9643,52 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>d5 Mon 06:45</t>
+          <t>d4 Sun 15:27</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>Amtrak Station</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>d5 Mon 13:56</t>
+          <t>d4 Sun 15:35</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Amtrak: Acela</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>7.18</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="L15" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>CT DE MA MD NJ NY PA RI</t>
-        </is>
-      </c>
+        <v>0.14</v>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="O15" t="inlineStr"/>
     </row>
@@ -9694,52 +9698,56 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>d5 Mon 13:56</t>
+          <t>d4 Sun 16:11</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>d5 Mon 14:04</t>
+          <t>d5 Mon 06:25</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Amtrak: Silver Meteor</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
+        <v>14.23</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="L16" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>GA NC SC VA</t>
+        </is>
+      </c>
       <c r="N16" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="O16" t="inlineStr"/>
     </row>
@@ -9754,61 +9762,53 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>d5 Mon 14:30</t>
+          <t>d5 Mon 06:45</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>d5 Mon 13:56</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>d5 Mon 17:00</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Hanover (Hanover Inn)</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Dartmouth Coach: Boston South Station -&gt; Hanover 14:30</t>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Amtrak: Acela</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>2.5</v>
+        <v>7.18</v>
       </c>
       <c r="K17" t="n">
-        <v>0.42</v>
+        <v>0.33</v>
       </c>
       <c r="L17" t="n">
         <v>1.5</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>CT DE MA MD NJ NY PA RI</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>25</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -9821,32 +9821,32 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>d5 Mon 17:00</t>
+          <t>d5 Mon 13:56</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Hanover (Hanover Inn)</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>d5 Mon 17:01</t>
+          <t>d5 Mon 14:04</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Main at Allen</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -9855,13 +9855,13 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0.03</v>
+        <v>0.15</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O18" t="inlineStr"/>
     </row>
@@ -9876,59 +9876,59 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>d5 Mon 17:10</t>
+          <t>d5 Mon 14:30</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Main at Allen</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>d5 Mon 17:00</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>NH</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>d5 Mon 17:38</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Sykes Ave @ Greyhound</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>VT</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Advance Transit: Yellow Route</t>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Dartmouth Coach: Boston South Station -&gt; Hanover 14:30</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="K19" s="5" t="n">
-        <v>0.14</v>
+        <v>2.5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.42</v>
       </c>
       <c r="L19" t="n">
         <v>1.5</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>VT</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="N19" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>tight</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
@@ -9943,32 +9943,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>d5 Mon 17:38</t>
+          <t>d5 Mon 17:00</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sykes Ave @ Greyhound</t>
+          <t>Hanover (Hanover Inn)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>VT</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>d5 Mon 17:38</t>
+          <t>d5 Mon 17:01</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>White River Junction Bus Station</t>
+          <t>Main at Allen</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>VT</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -9977,13 +9977,13 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O20" t="inlineStr"/>
     </row>
@@ -9998,49 +9998,53 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>d5 Mon 17:55</t>
+          <t>d5 Mon 17:10</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>White River Junction Bus Station</t>
+          <t>Main at Allen</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>d5 Mon 17:38</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Sykes Ave @ Greyhound</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>VT</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>d5 Mon 20:15</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Boston (South Station)</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Greyhound-us: Boston - Burlington - Montréal</t>
+          <t>Advance Transit: Yellow Route</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>2.33</v>
+        <v>0.47</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>0.27</v>
+        <v>0.14</v>
       </c>
       <c r="L21" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="M21" t="inlineStr"/>
+        <v>1.5</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
       <c r="N21" t="n">
         <v>26</v>
       </c>
@@ -10061,32 +10065,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>d5 Mon 20:15</t>
+          <t>d5 Mon 17:38</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Boston (South Station)</t>
+          <t>Sykes Ave @ Greyhound</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>VT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>d5 Mon 20:15</t>
+          <t>d5 Mon 17:38</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>White River Junction Bus Station</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>VT</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -10116,55 +10120,51 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>d5 Mon 20:25</t>
+          <t>d5 Mon 17:55</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>White River Junction Bus Station</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>d5 Mon 20:15</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Boston (South Station)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>d5 Mon 22:45</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Portland, ME</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
+          <t>Greyhound-us: Boston - Burlington - Montréal</t>
         </is>
       </c>
       <c r="J23" t="n">
         <v>2.33</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>0.15</v>
+        <v>0.27</v>
       </c>
       <c r="L23" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
+        <v>4.4</v>
+      </c>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -10183,32 +10183,32 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>d5 Mon 22:45</t>
+          <t>d5 Mon 20:15</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
+          <t>Boston (South Station)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>d5 Mon 23:04</t>
+          <t>d5 Mon 20:15</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>City of Portland</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -10217,13 +10217,13 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>0.33</v>
+        <v>0.01</v>
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O24" t="inlineStr"/>
     </row>
@@ -10238,53 +10238,61 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>d5 Mon 23:59</t>
+          <t>d5 Mon 20:25</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>City of Portland</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>d5 Mon 22:45</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>ME</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>d6 Tue 02:00</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Boston (South Station)</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>FlixBus-us: NYC - Boston - Portland - Bangor</t>
+          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0.91</v>
+        <v>2.33</v>
+      </c>
+      <c r="K25" s="5" t="n">
+        <v>0.15</v>
       </c>
       <c r="L25" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="M25" t="inlineStr"/>
+        <v>1.4</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
       <c r="N25" t="n">
         <v>27</v>
       </c>
-      <c r="O25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -10292,62 +10300,54 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>d6 Tue 02:15</t>
+          <t>d5 Mon 22:45</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Boston (South Station)</t>
+          <t>Portland, ME</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>d6 Tue 07:05</t>
+          <t>d5 Mon 23:04</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>New York Port Authority</t>
+          <t>City of Portland</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Greyhound-us: Boston - New York (Express Service)</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>4.83</v>
-      </c>
-      <c r="K26" s="5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L26" t="n">
-        <v>4</v>
-      </c>
+        <v>0.33</v>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="n">
         <v>27</v>
       </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>tight</t>
-        </is>
-      </c>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -10360,61 +10360,53 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>d6 Tue 09:55</t>
+          <t>d5 Mon 23:59</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>New York Port Authority</t>
+          <t>City of Portland</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>d7 Wed 04:10</t>
+          <t>d6 Tue 02:00</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>Boston (South Station)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Greyhound-us: New York - Pittsburgh - St. Louis</t>
+          <t>FlixBus-us: NYC - Boston - Portland - Bangor</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>18.25</v>
-      </c>
-      <c r="K27" s="6" t="n">
-        <v>2.83</v>
+        <v>2.02</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.91</v>
       </c>
       <c r="L27" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>IN OH WV</t>
-        </is>
-      </c>
+        <v>14.2</v>
+      </c>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="n">
-        <v>30</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>long wait</t>
-        </is>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -10427,57 +10419,57 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>d7 Wed 04:40</t>
+          <t>d6 Tue 02:15</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>Boston (South Station)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>d7 Wed 06:45</t>
+          <t>d6 Tue 07:05</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Louisville Bus Station</t>
+          <t>New York Port Authority</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Greyhound-us: Atlanta - Chicago</t>
+          <t>Greyhound-us: Boston - New York (Express Service)</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0.5</v>
+        <v>4.83</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>0.25</v>
       </c>
       <c r="L28" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="M28" t="inlineStr"/>
       <c r="N28" t="n">
-        <v>31</v>
-      </c>
-      <c r="O28" t="inlineStr"/>
+        <v>27</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -10490,22 +10482,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>d7 Wed 07:35</t>
+          <t>d6 Tue 09:55</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Louisville Bus Station</t>
+          <t>New York Port Authority</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>d7 Wed 09:30</t>
+          <t>d7 Wed 04:10</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -10520,23 +10512,31 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Greyhound-us: Atlanta - Chicago</t>
+          <t>Greyhound-us: New York - Pittsburgh - St. Louis</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0.83</v>
+        <v>18.25</v>
+      </c>
+      <c r="K29" s="6" t="n">
+        <v>2.83</v>
       </c>
       <c r="L29" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="M29" t="inlineStr"/>
+        <v>5.2</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>IN OH WV</t>
+        </is>
+      </c>
       <c r="N29" t="n">
-        <v>31</v>
-      </c>
-      <c r="O29" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>long wait</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -10544,12 +10544,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>d7 Wed 09:30</t>
+          <t>d7 Wed 04:40</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -10564,30 +10564,38 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>d7 Wed 09:30</t>
+          <t>d7 Wed 06:45</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Louisville Bus Station</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Greyhound-us: Atlanta - Chicago</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
+        <v>2.08</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L30" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="N30" t="n">
         <v>31</v>
       </c>
@@ -10604,57 +10612,53 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>d7 Wed 11:35</t>
+          <t>d7 Wed 07:35</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Louisville Bus Station</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>d7 Wed 09:30</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Indianapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>d7 Wed 14:40</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>South Bend</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Miller Transportation: Indianapolis -&gt; Elkhart</t>
+          <t>Greyhound-us: Atlanta - Chicago</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="K31" s="6" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="L31" s="4" t="n">
-        <v>24</v>
+        <v>1.92</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1.1</v>
       </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="n">
         <v>31</v>
       </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>long wait, daily anchor</t>
-        </is>
-      </c>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -10667,12 +10671,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>d7 Wed 14:40</t>
+          <t>d7 Wed 09:30</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>South Bend</t>
+          <t>Indianapolis Bus Station</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -10682,12 +10686,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>d7 Wed 14:41</t>
+          <t>d7 Wed 09:30</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -10701,7 +10705,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
@@ -10722,12 +10726,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>d7 Wed 15:24</t>
+          <t>d7 Wed 11:35</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -10737,12 +10741,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>d7 Wed 15:52</t>
+          <t>d7 Wed 14:40</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Adams &amp; Dylan</t>
+          <t>South Bend</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -10752,23 +10756,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Transpo (South Bend, IN): Blackthorn Express</t>
+          <t>Miller Transportation: Indianapolis -&gt; Elkhart</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="L33" t="n">
-        <v>2</v>
+        <v>3.08</v>
+      </c>
+      <c r="K33" s="6" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="L33" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="n">
         <v>31</v>
       </c>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>long wait, daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -10781,12 +10789,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>d7 Wed 15:52</t>
+          <t>d7 Wed 14:40</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Adams &amp; Dylan</t>
+          <t>South Bend</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -10796,17 +10804,17 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>d7 Wed 16:06</t>
+          <t>d7 Wed 14:41</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>MI state line (walk from Adams &amp; Dylan)</t>
+          <t>South Street Station</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -10815,17 +10823,13 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>0.24</v>
+        <v>0.03</v>
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>MI</t>
-        </is>
-      </c>
+      <c r="M34" t="inlineStr"/>
       <c r="N34" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O34" t="inlineStr"/>
     </row>
@@ -10835,27 +10839,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>d7 Wed 16:06</t>
+          <t>d7 Wed 15:24</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>MI state line (walk from Adams &amp; Dylan)</t>
+          <t>South Street Station</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>d7 Wed 16:20</t>
+          <t>d7 Wed 15:52</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -10870,17 +10874,21 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Transpo (South Bend, IN): Blackthorn Express</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+        <v>0.47</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L35" t="n">
+        <v>2</v>
+      </c>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O35" t="inlineStr"/>
     </row>
@@ -10890,12 +10898,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>d7 Wed 17:52</t>
+          <t>d7 Wed 15:52</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -10910,34 +10918,34 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>d7 Wed 18:28</t>
+          <t>d7 Wed 16:06</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>MI state line (walk from Adams &amp; Dylan)</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MI</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Transpo (South Bend, IN): Blackthorn Express</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K36" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="L36" t="n">
-        <v>14</v>
-      </c>
-      <c r="M36" t="inlineStr"/>
+        <v>0.24</v>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
       <c r="N36" t="n">
         <v>32</v>
       </c>
@@ -10954,41 +10962,41 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>d7 Wed 18:28</t>
+          <t>d7 Wed 16:06</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>MI state line (walk from Adams &amp; Dylan)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>d7 Wed 16:20</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Adams &amp; Dylan</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>d7 Wed 18:28</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>South Bend Transpo (S St Station)</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>walk / local</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>0.01</v>
+        <v>0.24</v>
       </c>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
@@ -11009,12 +11017,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>d7 Wed 18:55</t>
+          <t>d7 Wed 17:52</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>South Bend Transpo (S St Station)</t>
+          <t>Adams &amp; Dylan</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -11024,40 +11032,36 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>d7 Wed 20:05</t>
+          <t>d7 Wed 18:28</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>South Street Station</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Greyhound-us: Chicago - Cleveland - Washington</t>
+          <t>Transpo (South Bend, IN): Blackthorn Express</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>2.17</v>
+        <v>0.6</v>
       </c>
       <c r="K38" t="n">
-        <v>0.44</v>
+        <v>1.52</v>
       </c>
       <c r="L38" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O38" t="inlineStr"/>
     </row>
@@ -11067,60 +11071,52 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>d7 Wed 22:00</t>
+          <t>d7 Wed 18:28</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>South Street Station</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>d8 Thu 06:20</t>
+          <t>d7 Wed 18:28</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Minneapolis Bus Station</t>
+          <t>South Bend Transpo (S St Station)</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Greyhound-us: Chicago - Milwaukee - Minneapolis</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="K39" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="L39" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>MN WI</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
       <c r="N39" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="O39" t="inlineStr"/>
     </row>
@@ -11130,52 +11126,60 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>d8 Thu 06:20</t>
+          <t>d7 Wed 18:55</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Minneapolis Bus Station</t>
+          <t>South Bend Transpo (S St Station)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>d8 Thu 06:20</t>
+          <t>d7 Wed 20:05</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Greyhound-us: Chicago - Cleveland - Washington</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
+        <v>2.17</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L40" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
       <c r="N40" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O40" t="inlineStr"/>
     </row>
@@ -11190,61 +11194,57 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>d8 Thu 10:35</t>
+          <t>d7 Wed 22:00</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>d8 Thu 06:20</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Minneapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
           <t>MN</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>d8 Thu 14:55</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Fargo</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
+          <t>Greyhound-us: Chicago - Milwaukee - Minneapolis</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="K41" s="6" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="L41" s="4" t="n">
-        <v>24</v>
+        <v>8.33</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="L41" t="n">
+        <v>3.1</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>MN WI</t>
         </is>
       </c>
       <c r="N41" t="n">
-        <v>36</v>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>long wait, daily anchor</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -11252,66 +11252,54 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>d8 Thu 15:50</t>
+          <t>d8 Thu 06:20</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Fargo</t>
+          <t>Minneapolis Bus Station</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>d8 Thu 19:50</t>
+          <t>d8 Thu 06:20</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Fargo -&gt; Sioux Falls</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>4</v>
-      </c>
-      <c r="K42" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="L42" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
       <c r="N42" t="n">
-        <v>37</v>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -11324,59 +11312,59 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>d8 Thu 20:05</t>
+          <t>d8 Thu 10:35</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>d9 Fri 04:15</t>
+          <t>d8 Thu 14:55</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Sioux Falls -&gt; Kansas City</t>
+          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>8.17</v>
-      </c>
-      <c r="K43" s="5" t="n">
-        <v>0.25</v>
+        <v>4.33</v>
+      </c>
+      <c r="K43" s="6" t="n">
+        <v>4.24</v>
       </c>
       <c r="L43" s="4" t="n">
         <v>24</v>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>IA MO NE</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>tight, daily anchor</t>
+          <t>long wait, daily anchor</t>
         </is>
       </c>
     </row>
@@ -11386,54 +11374,66 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>d9 Fri 04:15</t>
+          <t>d8 Thu 15:50</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>d9 Fri 04:15</t>
+          <t>d8 Thu 19:50</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Kansas City Bus Station</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Jefferson Lines: Fargo -&gt; Sioux Falls</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L44" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
       <c r="N44" t="n">
-        <v>40</v>
-      </c>
-      <c r="O44" t="inlineStr"/>
+        <v>37</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -11446,59 +11446,59 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>d9 Fri 04:35</t>
+          <t>d8 Thu 20:05</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Kansas City Bus Station</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>d9 Fri 04:15</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Kansas City</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
           <t>MO</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>d9 Fri 16:05</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Denver Union Station Bus Concourse</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>CO</t>
-        </is>
-      </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Greyhound-us: St Louis - Denver</t>
+          <t>Jefferson Lines: Sioux Falls -&gt; Kansas City</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>12.5</v>
+        <v>8.17</v>
       </c>
       <c r="K45" s="5" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="L45" t="n">
-        <v>17.4</v>
+        <v>0.25</v>
+      </c>
+      <c r="L45" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>CO KS</t>
+          <t>IA MO NE</t>
         </is>
       </c>
       <c r="N45" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>tight</t>
+          <t>tight, daily anchor</t>
         </is>
       </c>
     </row>
@@ -11508,66 +11508,54 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>d9 Fri 16:35</t>
+          <t>d9 Fri 04:15</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Denver Union Station Bus Concourse</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>d10 Sat 14:30</t>
+          <t>d9 Fri 04:15</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Kansas City Bus Station</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Greyhound-us: Seattle-Boise-SLC-Denver</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>22.92</v>
-      </c>
-      <c r="K46" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L46" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>ID OR UT WA</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
       <c r="N46" t="n">
-        <v>46</v>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -11580,55 +11568,59 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>d10 Sat 14:40</t>
+          <t>d9 Fri 04:35</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Kansas City Bus Station</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>d10 Sat 17:00</t>
+          <t>d9 Fri 16:05</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Spokane Station</t>
+          <t>Denver Union Station Bus Concourse</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>FlixBus-us: Portland - Boise</t>
+          <t>Greyhound-us: St Louis - Denver</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>2.33</v>
+        <v>12.5</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="L47" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M47" t="inlineStr"/>
+        <v>0.32</v>
+      </c>
+      <c r="L47" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>CO KS</t>
+        </is>
+      </c>
       <c r="N47" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>tight, daily anchor</t>
+          <t>tight</t>
         </is>
       </c>
     </row>
@@ -11638,54 +11630,66 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>d10 Sat 17:00</t>
+          <t>d9 Fri 16:35</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Spokane Station</t>
+          <t>Denver Union Station Bus Concourse</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>d10 Sat 14:30</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>d10 Sat 17:00</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Spokane</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Greyhound-us: Seattle-Boise-SLC-Denver</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
+        <v>22.92</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L48" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>ID OR UT WA</t>
+        </is>
+      </c>
       <c r="N48" t="n">
         <v>46</v>
       </c>
-      <c r="O48" t="inlineStr"/>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -11698,12 +11702,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>d10 Sat 17:10</t>
+          <t>d10 Sat 14:40</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Spokane</t>
+          <t>Pasco Bus Stop</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -11713,40 +11717,36 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>d11 Sun 04:05</t>
+          <t>d10 Sat 17:00</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Billings</t>
+          <t>Spokane Station</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Spokane -&gt; Billings</t>
+          <t>FlixBus-us: Portland - Boise</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>9.92</v>
+        <v>2.33</v>
       </c>
       <c r="K49" s="5" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="L49" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
+      <c r="M49" t="inlineStr"/>
       <c r="N49" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -11760,62 +11760,184 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>d10 Sat 17:00</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Spokane Station</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>d10 Sat 17:00</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="n">
+        <v>46</v>
+      </c>
+      <c r="O50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>ride</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>d10 Sat 17:10</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>d11 Sun 04:05</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Spokane -&gt; Billings</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="K51" s="5" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="L51" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>47</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>tight, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
         <is>
           <t>d11 Sun 04:30</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>Billings</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>MT</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>d11 Sun 06:35</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>Sheridan WY Taco Bell 1655 Coffeen Ave (Jefferson)</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>WY</t>
         </is>
       </c>
-      <c r="I50" s="3" t="inlineStr">
+      <c r="I52" s="3" t="inlineStr">
         <is>
           <t>Jefferson Lines: JL 702 Billings -&gt; Sheridan (Nick screenshot Sep 22 2026: jeffersonlines.com 09/29 4:30 AM -&gt; 6:35 AM; feed trip 1632 skips Sheridan; daily assumed; Sheridan Taco Bell point approximate)</t>
         </is>
       </c>
-      <c r="J50" t="n">
+      <c r="J52" t="n">
         <v>2.08</v>
       </c>
-      <c r="K50" t="n">
+      <c r="K52" t="n">
         <v>0.42</v>
       </c>
-      <c r="L50" s="4" t="n">
+      <c r="L52" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>WY</t>
         </is>
       </c>
-      <c r="N50" t="n">
+      <c r="N52" t="n">
         <v>48</v>
       </c>
-      <c r="O50" t="inlineStr">
+      <c r="O52" t="inlineStr">
         <is>
           <t>manual, daily anchor</t>
         </is>

</xml_diff>

<commit_message>
RX: pin New Orleans and Mobile (20:50 via Biloxi, 03:45 to Tallahassee); same 234.75 h, bookable, no Lafayette backtrack
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/route_legs.xlsx
+++ b/docs/route_legs.xlsx
@@ -9341,7 +9341,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>d3 Sat 18:00</t>
+          <t>d3 Sat 20:50</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -9356,17 +9356,17 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>d3 Sat 21:15</t>
+          <t>d3 Sat 23:20</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Lafayette Transit System</t>
+          <t>Mobile Bus Station</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -9375,21 +9375,25 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="K10" s="5" t="n">
-        <v>0.17</v>
+        <v>2.5</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>3</v>
       </c>
       <c r="L10" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="M10" t="inlineStr"/>
+        <v>8.199999999999999</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
       <c r="N10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>tight</t>
+          <t>long wait</t>
         </is>
       </c>
     </row>
@@ -9404,17 +9408,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>d3 Sat 22:35</t>
+          <t>d4 Sun 03:45</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Lafayette Transit System</t>
+          <t>Mobile Bus Station</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -9438,17 +9442,17 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>11.42</v>
-      </c>
-      <c r="K11" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="L11" s="4" t="n">
-        <v>24</v>
+        <v>6.25</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="L11" t="n">
+        <v>5.4</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>AL FL</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="N11" t="n">
@@ -9456,7 +9460,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>daily anchor</t>
+          <t>long wait</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RX: Gulf leg as booked, Delta Bus Lines to Baton Rouge then the 23:55 through to Tallahassee; same 234.75 h
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/route_legs.xlsx
+++ b/docs/route_legs.xlsx
@@ -8839,7 +8839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9273,12 +9273,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>d3 Sat 08:50</t>
+          <t>d3 Sat 08:00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -9293,40 +9293,32 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>d3 Sat 17:50</t>
+          <t>d3 Sat 08:00</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>New Orleans Bus Station</t>
+          <t>Memphis (Airport)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Greyhound-us: Baton Rouge - New Orleans - Memphis</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>9</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="L9" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>LA MS</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O9" t="inlineStr"/>
     </row>
@@ -9341,59 +9333,59 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>d3 Sat 20:50</t>
+          <t>d3 Sat 10:00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>New Orleans Bus Station</t>
+          <t>Memphis (Airport)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>d3 Sat 18:30</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Baton Rouge</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>LA</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>d3 Sat 23:20</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Mobile Bus Station</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Greyhound-us: Atlanta - New Orleans - Houston</t>
+          <t>Delta Bus Lines Inc.: Memphis -&gt; Baton Rouge</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" t="n">
-        <v>8.199999999999999</v>
+        <v>8.5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>LA MS</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>long wait</t>
+          <t>daily anchor</t>
         </is>
       </c>
     </row>
@@ -9403,66 +9395,54 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>d4 Sun 03:45</t>
+          <t>d3 Sat 18:30</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Mobile Bus Station</t>
+          <t>Baton Rouge</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>d4 Sun 11:00</t>
+          <t>d3 Sat 18:30</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
+          <t>Baton Rouge Bus Station</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Greyhound-us: Orlando - Houston</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>4.42</v>
-      </c>
-      <c r="L11" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>12</v>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>long wait</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -9475,51 +9455,51 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>d4 Sun 11:25</t>
+          <t>d3 Sat 20:10</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
+          <t>Baton Rouge Bus Station</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>d4 Sun 14:50</t>
+          <t>d3 Sat 21:15</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Jacksonville (Downtown)</t>
+          <t>Lafayette Transit System</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Greyhound-us: Jacksonville - Mobile</t>
+          <t>Greyhound-us: Atlanta - New Orleans - Houston</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>3.42</v>
+        <v>1.08</v>
       </c>
       <c r="K12" t="n">
-        <v>0.42</v>
+        <v>1.66</v>
       </c>
       <c r="L12" t="n">
-        <v>5.8</v>
+        <v>0.8</v>
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O12" t="inlineStr"/>
     </row>
@@ -9529,54 +9509,66 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>d4 Sun 14:50</t>
+          <t>d3 Sat 22:35</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Jacksonville (Downtown)</t>
+          <t>Lafayette Transit System</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>d4 Sun 11:00</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>d4 Sun 14:50</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>JRTC Bay H</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Greyhound-us: Orlando - Houston</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
+        <v>11.42</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>AL FL</t>
+        </is>
+      </c>
       <c r="N13" t="n">
         <v>12</v>
       </c>
-      <c r="O13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -9589,12 +9581,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>d4 Sun 15:00</t>
+          <t>d4 Sun 11:25</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>JRTC Bay H</t>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -9604,12 +9596,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>d4 Sun 15:27</t>
+          <t>d4 Sun 14:50</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Amtrak Station</t>
+          <t>Jacksonville (Downtown)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -9619,27 +9611,23 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Jacksonville Transportation Authority: Kings Road</t>
+          <t>Greyhound-us: Jacksonville - Mobile</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="K14" s="5" t="n">
-        <v>0.15</v>
+        <v>3.42</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.42</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>5.8</v>
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
         <v>12</v>
       </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>tight</t>
-        </is>
-      </c>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9652,12 +9640,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>d4 Sun 15:27</t>
+          <t>d4 Sun 14:50</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Amtrak Station</t>
+          <t>Jacksonville (Downtown)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -9667,12 +9655,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>d4 Sun 15:35</t>
+          <t>d4 Sun 14:50</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>JRTC Bay H</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -9686,7 +9674,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>0.14</v>
+        <v>0.02</v>
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
@@ -9707,12 +9695,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>d4 Sun 16:11</t>
+          <t>d4 Sun 15:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>JRTC Bay H</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -9722,38 +9710,42 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>d5 Mon 06:25</t>
+          <t>d4 Sun 15:27</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
+          <t>Amtrak Station</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Amtrak: Silver Meteor</t>
+          <t>Jacksonville Transportation Authority: Kings Road</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>14.23</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0.59</v>
+        <v>0.45</v>
+      </c>
+      <c r="K16" s="5" t="n">
+        <v>0.15</v>
       </c>
       <c r="L16" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>GA NC SC VA</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
-        <v>16</v>
-      </c>
-      <c r="O16" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -9761,56 +9753,52 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>d5 Mon 06:45</t>
+          <t>d4 Sun 15:27</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>Amtrak Station</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>d5 Mon 13:56</t>
+          <t>d4 Sun 15:35</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Amtrak: Acela</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>7.18</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>CT DE MA MD NJ NY PA RI</t>
-        </is>
-      </c>
+        <v>0.14</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="O17" t="inlineStr"/>
     </row>
@@ -9820,52 +9808,56 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>d5 Mon 13:56</t>
+          <t>d4 Sun 16:11</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>d5 Mon 14:04</t>
+          <t>d5 Mon 06:25</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Amtrak: Silver Meteor</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
+        <v>14.23</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="L18" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>GA NC SC VA</t>
+        </is>
+      </c>
       <c r="N18" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="O18" t="inlineStr"/>
     </row>
@@ -9880,61 +9872,53 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>d5 Mon 14:30</t>
+          <t>d5 Mon 06:45</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>d5 Mon 13:56</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>d5 Mon 17:00</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Hanover (Hanover Inn)</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>Dartmouth Coach: Boston South Station -&gt; Hanover 14:30</t>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Amtrak: Acela</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>2.5</v>
+        <v>7.18</v>
       </c>
       <c r="K19" t="n">
-        <v>0.42</v>
+        <v>0.33</v>
       </c>
       <c r="L19" t="n">
         <v>1.5</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>CT DE MA MD NJ NY PA RI</t>
         </is>
       </c>
       <c r="N19" t="n">
-        <v>25</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9947,32 +9931,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>d5 Mon 17:00</t>
+          <t>d5 Mon 13:56</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Hanover (Hanover Inn)</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>d5 Mon 17:01</t>
+          <t>d5 Mon 14:04</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Main at Allen</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -9981,13 +9965,13 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>0.03</v>
+        <v>0.15</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O20" t="inlineStr"/>
     </row>
@@ -10002,59 +9986,59 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>d5 Mon 17:10</t>
+          <t>d5 Mon 14:30</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Main at Allen</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>d5 Mon 17:00</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>NH</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>d5 Mon 17:38</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Sykes Ave @ Greyhound</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>VT</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Advance Transit: Yellow Route</t>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Dartmouth Coach: Boston South Station -&gt; Hanover 14:30</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="K21" s="5" t="n">
-        <v>0.14</v>
+        <v>2.5</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.42</v>
       </c>
       <c r="L21" t="n">
         <v>1.5</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>VT</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>tight</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
@@ -10069,32 +10053,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>d5 Mon 17:38</t>
+          <t>d5 Mon 17:00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sykes Ave @ Greyhound</t>
+          <t>Hanover (Hanover Inn)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>VT</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>d5 Mon 17:38</t>
+          <t>d5 Mon 17:01</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>White River Junction Bus Station</t>
+          <t>Main at Allen</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>VT</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -10103,13 +10087,13 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O22" t="inlineStr"/>
     </row>
@@ -10124,49 +10108,53 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>d5 Mon 17:55</t>
+          <t>d5 Mon 17:10</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>White River Junction Bus Station</t>
+          <t>Main at Allen</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>d5 Mon 17:38</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Sykes Ave @ Greyhound</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>VT</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>d5 Mon 20:15</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Boston (South Station)</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Greyhound-us: Boston - Burlington - Montréal</t>
+          <t>Advance Transit: Yellow Route</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>2.33</v>
+        <v>0.47</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>0.27</v>
+        <v>0.14</v>
       </c>
       <c r="L23" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="M23" t="inlineStr"/>
+        <v>1.5</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
       <c r="N23" t="n">
         <v>26</v>
       </c>
@@ -10187,32 +10175,32 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>d5 Mon 20:15</t>
+          <t>d5 Mon 17:38</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Boston (South Station)</t>
+          <t>Sykes Ave @ Greyhound</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>VT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>d5 Mon 20:15</t>
+          <t>d5 Mon 17:38</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>White River Junction Bus Station</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>VT</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -10242,55 +10230,51 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>d5 Mon 20:25</t>
+          <t>d5 Mon 17:55</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>White River Junction Bus Station</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>d5 Mon 20:15</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Boston (South Station)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>d5 Mon 22:45</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Portland, ME</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
+          <t>Greyhound-us: Boston - Burlington - Montréal</t>
         </is>
       </c>
       <c r="J25" t="n">
         <v>2.33</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>0.15</v>
+        <v>0.27</v>
       </c>
       <c r="L25" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
+        <v>4.4</v>
+      </c>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -10309,32 +10293,32 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>d5 Mon 22:45</t>
+          <t>d5 Mon 20:15</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
+          <t>Boston (South Station)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>d5 Mon 23:04</t>
+          <t>d5 Mon 20:15</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>City of Portland</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -10343,13 +10327,13 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>0.33</v>
+        <v>0.01</v>
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O26" t="inlineStr"/>
     </row>
@@ -10364,53 +10348,61 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>d5 Mon 23:59</t>
+          <t>d5 Mon 20:25</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>City of Portland</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>d5 Mon 22:45</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
           <t>ME</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>d6 Tue 02:00</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Boston (South Station)</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>FlixBus-us: NYC - Boston - Portland - Bangor</t>
+          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0.91</v>
+        <v>2.33</v>
+      </c>
+      <c r="K27" s="5" t="n">
+        <v>0.15</v>
       </c>
       <c r="L27" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="M27" t="inlineStr"/>
+        <v>1.4</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
       <c r="N27" t="n">
         <v>27</v>
       </c>
-      <c r="O27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -10418,62 +10410,54 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>d6 Tue 02:15</t>
+          <t>d5 Mon 22:45</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Boston (South Station)</t>
+          <t>Portland, ME</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>d6 Tue 07:05</t>
+          <t>d5 Mon 23:04</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>New York Port Authority</t>
+          <t>City of Portland</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Greyhound-us: Boston - New York (Express Service)</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>4.83</v>
-      </c>
-      <c r="K28" s="5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L28" t="n">
-        <v>4</v>
-      </c>
+        <v>0.33</v>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="n">
         <v>27</v>
       </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>tight</t>
-        </is>
-      </c>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -10486,61 +10470,53 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>d6 Tue 09:55</t>
+          <t>d5 Mon 23:59</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>New York Port Authority</t>
+          <t>City of Portland</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>d7 Wed 04:10</t>
+          <t>d6 Tue 02:00</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>Boston (South Station)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Greyhound-us: New York - Pittsburgh - St. Louis</t>
+          <t>FlixBus-us: NYC - Boston - Portland - Bangor</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>18.25</v>
-      </c>
-      <c r="K29" s="6" t="n">
-        <v>2.83</v>
+        <v>2.02</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.91</v>
       </c>
       <c r="L29" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>IN OH WV</t>
-        </is>
-      </c>
+        <v>14.2</v>
+      </c>
+      <c r="M29" t="inlineStr"/>
       <c r="N29" t="n">
-        <v>30</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>long wait</t>
-        </is>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -10553,57 +10529,57 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>d7 Wed 04:40</t>
+          <t>d6 Tue 02:15</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>Boston (South Station)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>d7 Wed 06:45</t>
+          <t>d6 Tue 07:05</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Louisville Bus Station</t>
+          <t>New York Port Authority</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Greyhound-us: Atlanta - Chicago</t>
+          <t>Greyhound-us: Boston - New York (Express Service)</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0.5</v>
+        <v>4.83</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>0.25</v>
       </c>
       <c r="L30" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="M30" t="inlineStr"/>
       <c r="N30" t="n">
-        <v>31</v>
-      </c>
-      <c r="O30" t="inlineStr"/>
+        <v>27</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -10616,22 +10592,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>d7 Wed 07:35</t>
+          <t>d6 Tue 09:55</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Louisville Bus Station</t>
+          <t>New York Port Authority</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>d7 Wed 09:30</t>
+          <t>d7 Wed 04:10</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -10646,23 +10622,31 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Greyhound-us: Atlanta - Chicago</t>
+          <t>Greyhound-us: New York - Pittsburgh - St. Louis</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0.83</v>
+        <v>18.25</v>
+      </c>
+      <c r="K31" s="6" t="n">
+        <v>2.83</v>
       </c>
       <c r="L31" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="M31" t="inlineStr"/>
+        <v>5.2</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>IN OH WV</t>
+        </is>
+      </c>
       <c r="N31" t="n">
-        <v>31</v>
-      </c>
-      <c r="O31" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>long wait</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -10670,12 +10654,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>d7 Wed 09:30</t>
+          <t>d7 Wed 04:40</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -10690,30 +10674,38 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>d7 Wed 09:30</t>
+          <t>d7 Wed 06:45</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Louisville Bus Station</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Greyhound-us: Atlanta - Chicago</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+        <v>2.08</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L32" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="N32" t="n">
         <v>31</v>
       </c>
@@ -10730,57 +10722,53 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>d7 Wed 11:35</t>
+          <t>d7 Wed 07:35</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Louisville Bus Station</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>d7 Wed 09:30</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Indianapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>d7 Wed 14:40</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>South Bend</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Miller Transportation: Indianapolis -&gt; Elkhart</t>
+          <t>Greyhound-us: Atlanta - Chicago</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="K33" s="6" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="L33" s="4" t="n">
-        <v>24</v>
+        <v>1.92</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1.1</v>
       </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="n">
         <v>31</v>
       </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>long wait, daily anchor</t>
-        </is>
-      </c>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -10793,12 +10781,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>d7 Wed 14:40</t>
+          <t>d7 Wed 09:30</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>South Bend</t>
+          <t>Indianapolis Bus Station</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -10808,12 +10796,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>d7 Wed 14:41</t>
+          <t>d7 Wed 09:30</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -10827,7 +10815,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -10848,12 +10836,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>d7 Wed 15:24</t>
+          <t>d7 Wed 11:35</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -10863,12 +10851,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>d7 Wed 15:52</t>
+          <t>d7 Wed 14:40</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Adams &amp; Dylan</t>
+          <t>South Bend</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -10878,23 +10866,27 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Transpo (South Bend, IN): Blackthorn Express</t>
+          <t>Miller Transportation: Indianapolis -&gt; Elkhart</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="L35" t="n">
-        <v>2</v>
+        <v>3.08</v>
+      </c>
+      <c r="K35" s="6" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="L35" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="n">
         <v>31</v>
       </c>
-      <c r="O35" t="inlineStr"/>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>long wait, daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -10907,12 +10899,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>d7 Wed 15:52</t>
+          <t>d7 Wed 14:40</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Adams &amp; Dylan</t>
+          <t>South Bend</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -10922,17 +10914,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>d7 Wed 16:06</t>
+          <t>d7 Wed 14:41</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>MI state line (walk from Adams &amp; Dylan)</t>
+          <t>South Street Station</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -10941,17 +10933,13 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>0.24</v>
+        <v>0.03</v>
       </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>MI</t>
-        </is>
-      </c>
+      <c r="M36" t="inlineStr"/>
       <c r="N36" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O36" t="inlineStr"/>
     </row>
@@ -10961,27 +10949,27 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>d7 Wed 16:06</t>
+          <t>d7 Wed 15:24</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>MI state line (walk from Adams &amp; Dylan)</t>
+          <t>South Street Station</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>d7 Wed 16:20</t>
+          <t>d7 Wed 15:52</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -10996,17 +10984,21 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Transpo (South Bend, IN): Blackthorn Express</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+        <v>0.47</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L37" t="n">
+        <v>2</v>
+      </c>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O37" t="inlineStr"/>
     </row>
@@ -11016,12 +11008,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>d7 Wed 17:52</t>
+          <t>d7 Wed 15:52</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -11036,34 +11028,34 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>d7 Wed 18:28</t>
+          <t>d7 Wed 16:06</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>MI state line (walk from Adams &amp; Dylan)</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MI</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Transpo (South Bend, IN): Blackthorn Express</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K38" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="L38" t="n">
-        <v>14</v>
-      </c>
-      <c r="M38" t="inlineStr"/>
+        <v>0.24</v>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
       <c r="N38" t="n">
         <v>32</v>
       </c>
@@ -11080,41 +11072,41 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>d7 Wed 18:28</t>
+          <t>d7 Wed 16:06</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>MI state line (walk from Adams &amp; Dylan)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>d7 Wed 16:20</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Adams &amp; Dylan</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>d7 Wed 18:28</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>South Bend Transpo (S St Station)</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>walk / local</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>0.01</v>
+        <v>0.24</v>
       </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
@@ -11135,12 +11127,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>d7 Wed 18:55</t>
+          <t>d7 Wed 17:52</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>South Bend Transpo (S St Station)</t>
+          <t>Adams &amp; Dylan</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -11150,40 +11142,36 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>d7 Wed 20:05</t>
+          <t>d7 Wed 18:28</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>South Street Station</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Greyhound-us: Chicago - Cleveland - Washington</t>
+          <t>Transpo (South Bend, IN): Blackthorn Express</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>2.17</v>
+        <v>0.6</v>
       </c>
       <c r="K40" t="n">
-        <v>0.44</v>
+        <v>1.52</v>
       </c>
       <c r="L40" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O40" t="inlineStr"/>
     </row>
@@ -11193,60 +11181,52 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>d7 Wed 22:00</t>
+          <t>d7 Wed 18:28</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>South Street Station</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>d8 Thu 06:20</t>
+          <t>d7 Wed 18:28</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Minneapolis Bus Station</t>
+          <t>South Bend Transpo (S St Station)</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Greyhound-us: Chicago - Milwaukee - Minneapolis</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="K41" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="L41" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>MN WI</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
       <c r="N41" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="O41" t="inlineStr"/>
     </row>
@@ -11256,52 +11236,60 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>d8 Thu 06:20</t>
+          <t>d7 Wed 18:55</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Minneapolis Bus Station</t>
+          <t>South Bend Transpo (S St Station)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>d8 Thu 06:20</t>
+          <t>d7 Wed 20:05</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Greyhound-us: Chicago - Cleveland - Washington</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
+        <v>2.17</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L42" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
       <c r="N42" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O42" t="inlineStr"/>
     </row>
@@ -11316,61 +11304,57 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>d8 Thu 10:35</t>
+          <t>d7 Wed 22:00</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>d8 Thu 06:20</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Minneapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
           <t>MN</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>d8 Thu 14:55</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Fargo</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
+          <t>Greyhound-us: Chicago - Milwaukee - Minneapolis</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="K43" s="6" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="L43" s="4" t="n">
-        <v>24</v>
+        <v>8.33</v>
+      </c>
+      <c r="K43" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="L43" t="n">
+        <v>3.1</v>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>MN WI</t>
         </is>
       </c>
       <c r="N43" t="n">
-        <v>36</v>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>long wait, daily anchor</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -11378,66 +11362,54 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>d8 Thu 15:50</t>
+          <t>d8 Thu 06:20</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Fargo</t>
+          <t>Minneapolis Bus Station</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>d8 Thu 19:50</t>
+          <t>d8 Thu 06:20</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Fargo -&gt; Sioux Falls</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>4</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="L44" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
       <c r="N44" t="n">
-        <v>37</v>
-      </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -11450,59 +11422,59 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>d8 Thu 20:05</t>
+          <t>d8 Thu 10:35</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>d9 Fri 04:15</t>
+          <t>d8 Thu 14:55</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Sioux Falls -&gt; Kansas City</t>
+          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>8.17</v>
-      </c>
-      <c r="K45" s="5" t="n">
-        <v>0.25</v>
+        <v>4.33</v>
+      </c>
+      <c r="K45" s="6" t="n">
+        <v>4.24</v>
       </c>
       <c r="L45" s="4" t="n">
         <v>24</v>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>IA MO NE</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>tight, daily anchor</t>
+          <t>long wait, daily anchor</t>
         </is>
       </c>
     </row>
@@ -11512,54 +11484,66 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>d9 Fri 04:15</t>
+          <t>d8 Thu 15:50</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>d9 Fri 04:15</t>
+          <t>d8 Thu 19:50</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Kansas City Bus Station</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Jefferson Lines: Fargo -&gt; Sioux Falls</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L46" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
       <c r="N46" t="n">
-        <v>40</v>
-      </c>
-      <c r="O46" t="inlineStr"/>
+        <v>37</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -11572,59 +11556,59 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>d9 Fri 04:35</t>
+          <t>d8 Thu 20:05</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Kansas City Bus Station</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>d9 Fri 04:15</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Kansas City</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
           <t>MO</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>d9 Fri 16:05</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Denver Union Station Bus Concourse</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>CO</t>
-        </is>
-      </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Greyhound-us: St Louis - Denver</t>
+          <t>Jefferson Lines: Sioux Falls -&gt; Kansas City</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>12.5</v>
+        <v>8.17</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="L47" t="n">
-        <v>17.4</v>
+        <v>0.25</v>
+      </c>
+      <c r="L47" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>CO KS</t>
+          <t>IA MO NE</t>
         </is>
       </c>
       <c r="N47" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>tight</t>
+          <t>tight, daily anchor</t>
         </is>
       </c>
     </row>
@@ -11634,66 +11618,54 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>d9 Fri 16:35</t>
+          <t>d9 Fri 04:15</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Denver Union Station Bus Concourse</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>d10 Sat 14:30</t>
+          <t>d9 Fri 04:15</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Kansas City Bus Station</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Greyhound-us: Seattle-Boise-SLC-Denver</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>22.92</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L48" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>ID OR UT WA</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
       <c r="N48" t="n">
-        <v>46</v>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -11706,55 +11678,59 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>d10 Sat 14:40</t>
+          <t>d9 Fri 04:35</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Kansas City Bus Station</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>d10 Sat 17:00</t>
+          <t>d9 Fri 16:05</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Spokane Station</t>
+          <t>Denver Union Station Bus Concourse</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>FlixBus-us: Portland - Boise</t>
+          <t>Greyhound-us: St Louis - Denver</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>2.33</v>
+        <v>12.5</v>
       </c>
       <c r="K49" s="5" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="L49" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M49" t="inlineStr"/>
+        <v>0.32</v>
+      </c>
+      <c r="L49" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>CO KS</t>
+        </is>
+      </c>
       <c r="N49" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>tight, daily anchor</t>
+          <t>tight</t>
         </is>
       </c>
     </row>
@@ -11764,54 +11740,66 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>d10 Sat 17:00</t>
+          <t>d9 Fri 16:35</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Spokane Station</t>
+          <t>Denver Union Station Bus Concourse</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>d10 Sat 14:30</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>d10 Sat 17:00</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Spokane</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Greyhound-us: Seattle-Boise-SLC-Denver</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
+        <v>22.92</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L50" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>ID OR UT WA</t>
+        </is>
+      </c>
       <c r="N50" t="n">
         <v>46</v>
       </c>
-      <c r="O50" t="inlineStr"/>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -11824,12 +11812,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>d10 Sat 17:10</t>
+          <t>d10 Sat 14:40</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Spokane</t>
+          <t>Pasco Bus Stop</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -11839,40 +11827,36 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>d11 Sun 04:05</t>
+          <t>d10 Sat 17:00</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Billings</t>
+          <t>Spokane Station</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Spokane -&gt; Billings</t>
+          <t>FlixBus-us: Portland - Boise</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>9.92</v>
+        <v>2.33</v>
       </c>
       <c r="K51" s="5" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="L51" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
+      <c r="M51" t="inlineStr"/>
       <c r="N51" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
@@ -11886,62 +11870,184 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>d10 Sat 17:00</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Spokane Station</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>d10 Sat 17:00</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="n">
+        <v>46</v>
+      </c>
+      <c r="O52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>ride</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>d10 Sat 17:10</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>d11 Sun 04:05</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Spokane -&gt; Billings</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="K53" s="5" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="L53" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>47</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>tight, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
         <is>
           <t>d11 Sun 04:30</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>Billings</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>MT</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>d11 Sun 06:35</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>Sheridan WY Taco Bell 1655 Coffeen Ave (Jefferson)</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>WY</t>
         </is>
       </c>
-      <c r="I52" s="3" t="inlineStr">
+      <c r="I54" s="3" t="inlineStr">
         <is>
           <t>Jefferson Lines: JL 702 Billings -&gt; Sheridan (Nick screenshot Sep 22 2026: jeffersonlines.com 09/29 4:30 AM -&gt; 6:35 AM; feed trip 1632 skips Sheridan; daily assumed; Sheridan Taco Bell point approximate)</t>
         </is>
       </c>
-      <c r="J52" t="n">
+      <c r="J54" t="n">
         <v>2.08</v>
       </c>
-      <c r="K52" t="n">
+      <c r="K54" t="n">
         <v>0.42</v>
       </c>
-      <c r="L52" s="4" t="n">
+      <c r="L54" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>WY</t>
         </is>
       </c>
-      <c r="N52" t="n">
+      <c r="N54" t="n">
         <v>48</v>
       </c>
-      <c r="O52" t="inlineStr">
+      <c r="O54" t="inlineStr">
         <is>
           <t>manual, daily anchor</t>
         </is>

</xml_diff>

<commit_message>
Measured walk links now collect their state (TimeRouter.walk_collects); South Sioux City walk; Sioux City Transit
The guard against collecting a state by walking into a real stop also caught the end points of
data/walk_links.csv, and coverage only counted walks to virtual walk-in points, so no hand-measured
border walk (Big River Crossing, Michiana, the Vermont runs, East Dubuque, now South Sioux City)
could ever collect its state. walk_collects is now the one rule, used by time_search, ride_search
and route_sheets; _crosses exempts link end points. New regress check fails without it (13/13).
Control replay: same 29/39, every rank unchanged; leg 5 menu 78 -> 79 (Big River Crossing).
All six routes unchanged. Sheridan -> Sioux City/Nebraska bank: 239.17 h.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/route_legs.xlsx
+++ b/docs/route_legs.xlsx
@@ -10737,12 +10737,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>d7 Wed 09:30</t>
+          <t>d7 Wed 12:35</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>Gary Bus Station</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -10756,19 +10756,23 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>1.92</v>
+        <v>6</v>
       </c>
       <c r="K33" t="n">
         <v>0.83</v>
       </c>
-      <c r="L33" t="n">
-        <v>1.1</v>
+      <c r="L33" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="n">
         <v>31</v>
       </c>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -10781,12 +10785,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>d7 Wed 09:30</t>
+          <t>d7 Wed 12:35</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>Gary Bus Station</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -10796,12 +10800,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>d7 Wed 09:30</t>
+          <t>d7 Wed 12:36</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Gary Metro Center</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -10815,7 +10819,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -10836,12 +10840,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>d7 Wed 11:35</t>
+          <t>d7 Wed 12:50</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Gary Metro Center</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -10851,12 +10855,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>d7 Wed 14:40</t>
+          <t>d7 Wed 13:04</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>South Bend</t>
+          <t>Hammond Gateway</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -10866,17 +10870,17 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Miller Transportation: Indianapolis -&gt; Elkhart</t>
+          <t>Northern Indiana Commuter Transportation District: Lakeshore Corridor</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="K35" s="6" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="L35" s="4" t="n">
-        <v>24</v>
+        <v>0.23</v>
+      </c>
+      <c r="K35" s="5" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1.1</v>
       </c>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="n">
@@ -10884,7 +10888,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>long wait, daily anchor</t>
+          <t>tight</t>
         </is>
       </c>
     </row>
@@ -10894,17 +10898,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>d7 Wed 14:40</t>
+          <t>d7 Wed 13:14</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>South Bend</t>
+          <t>Hammond Gateway</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -10914,12 +10918,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>d7 Wed 14:41</t>
+          <t>d7 Wed 13:57</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>11th St. (Michigan City)</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -10929,19 +10933,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Northern Indiana Commuter Transportation District: Lakeshore Corridor</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+        <v>0.72</v>
+      </c>
+      <c r="K36" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1.1</v>
+      </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="n">
         <v>31</v>
       </c>
-      <c r="O36" t="inlineStr"/>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -10949,17 +10961,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>d7 Wed 15:24</t>
+          <t>d7 Wed 13:57</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>11th St. (Michigan City)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -10969,12 +10981,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>d7 Wed 15:52</t>
+          <t>d7 Wed 14:13</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Adams &amp; Dylan</t>
+          <t xml:space="preserve">E 4th Street/Franklin Street                                       </t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -10984,18 +10996,14 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Transpo (South Bend, IN): Blackthorn Express</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="K37" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="L37" t="n">
-        <v>2</v>
-      </c>
+        <v>0.27</v>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="n">
         <v>31</v>
@@ -11008,17 +11016,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>d7 Wed 15:52</t>
+          <t>d7 Wed 14:51</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Adams &amp; Dylan</t>
+          <t xml:space="preserve">E 4th Street/Franklin Street                                       </t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -11028,36 +11036,36 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>d7 Wed 16:06</t>
+          <t>d7 Wed 15:09</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>MI state line (walk from Adams &amp; Dylan)</t>
+          <t>Als Karwick</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Michian City Transit: Franklin St./Washington Park/Lakeland/Karwick</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>MI</t>
-        </is>
-      </c>
+        <v>0.3</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="L38" t="n">
+        <v>1</v>
+      </c>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O38" t="inlineStr"/>
     </row>
@@ -11072,45 +11080,49 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>d7 Wed 16:06</t>
+          <t>d7 Wed 15:09</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>MI state line (walk from Adams &amp; Dylan)</t>
+          <t>Als Karwick</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>d7 Wed 17:00</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Michigan line at Michiana (on foot from Michigan City Carroll Ave)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
           <t>MI</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>d7 Wed 16:20</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Adams &amp; Dylan</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>walk / local</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>0.24</v>
+        <v>0.85</v>
       </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
       <c r="N39" t="n">
         <v>32</v>
       </c>
@@ -11122,53 +11134,49 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>d7 Wed 17:52</t>
+          <t>d7 Wed 17:00</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Adams &amp; Dylan</t>
+          <t>Michigan line at Michiana (on foot from Michigan City Carroll Ave)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>d7 Wed 17:25</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Carroll Ave. (Michigan City)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>d7 Wed 18:28</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>South Street Station</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Transpo (South Bend, IN): Blackthorn Express</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K40" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="L40" t="n">
-        <v>14</v>
-      </c>
+        <v>1.42</v>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="n">
         <v>32</v>
@@ -11181,17 +11189,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>d7 Wed 18:28</t>
+          <t>d7 Wed 17:39</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>South Street Station</t>
+          <t>Carroll Ave. (Michigan City)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -11201,34 +11209,46 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>d7 Wed 18:28</t>
+          <t>d7 Wed 18:57</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>South Bend Transpo (S St Station)</t>
+          <t>Museum Campus/11th St.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Northern Indiana Commuter Transportation District: Lakeshore Corridor</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
+        <v>1.3</v>
+      </c>
+      <c r="K41" s="5" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="L41" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
       <c r="N41" t="n">
-        <v>32</v>
-      </c>
-      <c r="O41" t="inlineStr"/>
+        <v>33</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -11236,27 +11256,27 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>d7 Wed 18:55</t>
+          <t>d7 Wed 18:57</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>South Bend Transpo (S St Station)</t>
+          <t>Museum Campus/11th St.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>d7 Wed 20:05</t>
+          <t>d7 Wed 19:34</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -11271,23 +11291,15 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Greyhound-us: Chicago - Cleveland - Washington</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>2.17</v>
-      </c>
-      <c r="K42" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="L42" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
+        <v>0.63</v>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
       <c r="N42" t="n">
         <v>33</v>
       </c>
@@ -11340,8 +11352,8 @@
       <c r="J43" t="n">
         <v>8.33</v>
       </c>
-      <c r="K43" t="n">
-        <v>1.92</v>
+      <c r="K43" s="6" t="n">
+        <v>2.42</v>
       </c>
       <c r="L43" t="n">
         <v>3.1</v>
@@ -11354,7 +11366,11 @@
       <c r="N43" t="n">
         <v>35</v>
       </c>
-      <c r="O43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>long wait</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -19624,7 +19640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O67"/>
+  <dimension ref="A1:O70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -22600,12 +22616,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>d11 Sun 09:30</t>
+          <t>d11 Sun 12:35</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>Gary Bus Station</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -22619,19 +22635,23 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>1.92</v>
+        <v>6</v>
       </c>
       <c r="K51" t="n">
         <v>0.83</v>
       </c>
-      <c r="L51" t="n">
-        <v>1.1</v>
+      <c r="L51" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="n">
         <v>36</v>
       </c>
-      <c r="O51" t="inlineStr"/>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -22644,12 +22664,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>d11 Sun 09:30</t>
+          <t>d11 Sun 12:35</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>Gary Bus Station</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -22659,12 +22679,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>d11 Sun 09:30</t>
+          <t>d11 Sun 12:36</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Gary Metro Center</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -22678,7 +22698,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
@@ -22699,12 +22719,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>d11 Sun 10:50</t>
+          <t>d11 Sun 13:31</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Gary Metro Center</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -22714,46 +22734,38 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>d11 Sun 15:55</t>
+          <t>d11 Sun 13:41</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>East Chicago</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Barons Bus Lines: Cincinnati (Greyhound) -&gt; Detroit</t>
+          <t>Northern Indiana Commuter Transportation District: Lakeshore Corridor</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>5.08</v>
+        <v>0.17</v>
       </c>
       <c r="K53" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="L53" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>MI</t>
-        </is>
-      </c>
+        <v>0.91</v>
+      </c>
+      <c r="L53" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="M53" t="inlineStr"/>
       <c r="N53" t="n">
-        <v>37</v>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -22761,54 +22773,62 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>d11 Sun 15:55</t>
+          <t>d11 Sun 13:53</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>East Chicago</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>d11 Sun 15:55</t>
+          <t>d11 Sun 14:36</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Detroit Bus Station</t>
+          <t>Carroll Ave. (Michigan City)</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Northern Indiana Commuter Transportation District: Lakeshore Corridor</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+        <v>0.72</v>
+      </c>
+      <c r="K54" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L54" t="n">
+        <v>2.4</v>
+      </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="n">
-        <v>37</v>
-      </c>
-      <c r="O54" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -22816,60 +22836,56 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>d11 Sun 16:20</t>
+          <t>d11 Sun 14:36</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Detroit Bus Station</t>
+          <t>Carroll Ave. (Michigan City)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>d11 Sun 17:01</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Michigan line at Michiana (on foot from Michigan City Carroll Ave)</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
           <t>MI</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>d11 Sun 21:25</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>Chicago Bus Station</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Greyhound-us: Chicago - Kalamazoo - Detroit</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="K55" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="L55" t="n">
-        <v>8</v>
-      </c>
+        <v>1.42</v>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MI</t>
         </is>
       </c>
       <c r="N55" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O55" t="inlineStr"/>
     </row>
@@ -22879,60 +22895,52 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>d11 Sun 22:00</t>
+          <t>d11 Sun 17:01</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>Michigan line at Michiana (on foot from Michigan City Carroll Ave)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MI</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>d12 Mon 06:20</t>
+          <t>d11 Sun 17:26</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Minneapolis Bus Station</t>
+          <t>Carroll Ave. (Michigan City)</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Greyhound-us: Chicago - Milwaukee - Minneapolis</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J56" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="K56" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="L56" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>MN WI</t>
-        </is>
-      </c>
+        <v>1.42</v>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
       <c r="N56" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="O56" t="inlineStr"/>
     </row>
@@ -22942,52 +22950,60 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>d12 Mon 06:20</t>
+          <t>d11 Sun 19:05</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Minneapolis Bus Station</t>
+          <t>Carroll Ave. (Michigan City)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>d12 Mon 06:20</t>
+          <t>d11 Sun 20:29</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Museum Campus/11th St.</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Northern Indiana Commuter Transportation District: Lakeshore Corridor</t>
         </is>
       </c>
       <c r="J57" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
+        <v>1.4</v>
+      </c>
+      <c r="K57" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="L57" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
       <c r="N57" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="O57" t="inlineStr"/>
     </row>
@@ -22997,66 +23013,54 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>d12 Mon 10:35</t>
+          <t>d11 Sun 20:29</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Museum Campus/11th St.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>d12 Mon 14:55</t>
+          <t>d11 Sun 21:06</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Fargo</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J58" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="K58" s="6" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="L58" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
+        <v>0.63</v>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
       <c r="N58" t="n">
-        <v>41</v>
-      </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>long wait, daily anchor</t>
-        </is>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -23069,57 +23073,55 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>d12 Mon 15:50</t>
+          <t>d11 Sun 22:00</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Fargo</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>d12 Mon 19:50</t>
+          <t>d12 Mon 06:20</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Minneapolis Bus Station</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Fargo -&gt; Sioux Falls</t>
+          <t>Greyhound-us: Chicago - Milwaukee - Minneapolis</t>
         </is>
       </c>
       <c r="J59" t="n">
-        <v>4</v>
+        <v>8.33</v>
       </c>
       <c r="K59" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>none in 72 h</t>
-        </is>
+        <v>0.89</v>
+      </c>
+      <c r="L59" t="n">
+        <v>3.1</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MN WI</t>
         </is>
       </c>
       <c r="N59" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O59" t="inlineStr"/>
     </row>
@@ -23129,66 +23131,54 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>d12 Mon 20:05</t>
+          <t>d12 Mon 06:20</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Minneapolis Bus Station</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>d13 Tue 04:15</t>
+          <t>d12 Mon 06:20</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Sioux Falls -&gt; Kansas City</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J60" t="n">
-        <v>8.17</v>
-      </c>
-      <c r="K60" s="5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L60" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>IA MO NE</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
       <c r="N60" t="n">
-        <v>45</v>
-      </c>
-      <c r="O60" t="inlineStr">
-        <is>
-          <t>tight, daily anchor</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -23201,59 +23191,59 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>d13 Tue 08:20</t>
+          <t>d12 Mon 10:35</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>d13 Tue 12:30</t>
+          <t>d12 Mon 14:55</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Fayetteville</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Kansas City -&gt; Texarkana</t>
+          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>4.17</v>
+        <v>4.33</v>
       </c>
       <c r="K61" s="6" t="n">
-        <v>4.08</v>
-      </c>
-      <c r="L61" t="n">
-        <v>13.9</v>
+        <v>4.24</v>
+      </c>
+      <c r="L61" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="N61" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>long wait</t>
+          <t>long wait, daily anchor</t>
         </is>
       </c>
     </row>
@@ -23268,61 +23258,59 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>d13 Tue 13:35</t>
+          <t>d12 Mon 15:50</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Fayetteville</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>d13 Tue 20:05</t>
+          <t>d12 Mon 19:50</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Memphis (MATA Airways Transit Center)</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Tulsa -&gt; Memphis</t>
+          <t>Jefferson Lines: Fargo -&gt; Sioux Falls</t>
         </is>
       </c>
       <c r="J62" t="n">
-        <v>6.5</v>
+        <v>4</v>
       </c>
       <c r="K62" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="L62" s="4" t="n">
-        <v>24</v>
+        <v>0.92</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>none in 72 h</t>
+        </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="N62" t="n">
-        <v>47</v>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -23330,54 +23318,66 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>d13 Tue 20:05</t>
+          <t>d12 Mon 20:05</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Memphis (MATA Airways Transit Center)</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>d13 Tue 20:12</t>
+          <t>d13 Tue 04:15</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>AIRWAYS BOULEVARD at BROOKS ROAD</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Jefferson Lines: Sioux Falls -&gt; Kansas City</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
+        <v>8.17</v>
+      </c>
+      <c r="K63" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L63" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>IA MO NE</t>
+        </is>
+      </c>
       <c r="N63" t="n">
-        <v>47</v>
-      </c>
-      <c r="O63" t="inlineStr"/>
+        <v>45</v>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>tight, daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -23390,55 +23390,59 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>d13 Tue 20:19</t>
+          <t>d13 Tue 08:20</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>AIRWAYS BOULEVARD at BROOKS ROAD</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>d13 Tue 20:26</t>
+          <t>d13 Tue 12:30</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>BROOKS ROAD at COUGHLIN DRIVE</t>
+          <t>Fayetteville</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>MATA: BROOKS</t>
+          <t>Jefferson Lines: Kansas City -&gt; Texarkana</t>
         </is>
       </c>
       <c r="J64" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="K64" s="5" t="n">
-        <v>0.12</v>
+        <v>4.17</v>
+      </c>
+      <c r="K64" s="6" t="n">
+        <v>4.08</v>
       </c>
       <c r="L64" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="M64" t="inlineStr"/>
+        <v>13.9</v>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
       <c r="N64" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>tight</t>
+          <t>long wait</t>
         </is>
       </c>
     </row>
@@ -23448,54 +23452,66 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>d13 Tue 20:26</t>
+          <t>d13 Tue 13:35</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>BROOKS ROAD at COUGHLIN DRIVE</t>
+          <t>Fayetteville</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>d13 Tue 20:05</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Memphis (MATA Airways Transit Center)</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
           <t>TN</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>d13 Tue 20:44</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>ELVIS PRESLEY BLVD at SPRINGBROOK AVENUE</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Tulsa -&gt; Memphis</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="K65" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="L65" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M65" t="inlineStr">
         <is>
           <t>TN</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>walk / local</t>
-        </is>
-      </c>
-      <c r="J65" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
       <c r="N65" t="n">
         <v>47</v>
       </c>
-      <c r="O65" t="inlineStr"/>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -23503,17 +23519,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>d13 Tue 20:51</t>
+          <t>d13 Tue 20:05</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ELVIS PRESLEY BLVD at SPRINGBROOK AVENUE</t>
+          <t>Memphis (MATA Airways Transit Center)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -23523,12 +23539,12 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>d13 Tue 21:07</t>
+          <t>d13 Tue 20:12</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>HOLMES at ELVIS PRESLEY</t>
+          <t>AIRWAYS BOULEVARD at BROOKS ROAD</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -23538,27 +23554,19 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>MATA: CROSSTOWN</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J66" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="K66" s="5" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="L66" t="n">
-        <v>8</v>
-      </c>
+        <v>0.13</v>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr"/>
       <c r="N66" t="n">
         <v>47</v>
       </c>
-      <c r="O66" t="inlineStr">
-        <is>
-          <t>tight</t>
-        </is>
-      </c>
+      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -23566,58 +23574,239 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>d13 Tue 20:19</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>AIRWAYS BOULEVARD at BROOKS ROAD</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>d13 Tue 20:26</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>BROOKS ROAD at COUGHLIN DRIVE</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>MATA: BROOKS</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="K67" s="5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="L67" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="n">
+        <v>47</v>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>65</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>walk</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>d13 Tue 20:26</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>BROOKS ROAD at COUGHLIN DRIVE</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>d13 Tue 20:44</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>ELVIS PRESLEY BLVD at SPRINGBROOK AVENUE</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="n">
+        <v>47</v>
+      </c>
+      <c r="O68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>66</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>d13 Tue 20:51</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>ELVIS PRESLEY BLVD at SPRINGBROOK AVENUE</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
         <is>
           <t>d13 Tue 21:07</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>HOLMES at ELVIS PRESLEY</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
+      <c r="H69" t="inlineStr">
         <is>
           <t>TN</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>MATA: CROSSTOWN</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K69" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="L69" t="n">
+        <v>8</v>
+      </c>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="n">
+        <v>47</v>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>67</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>d13 Tue 21:07</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>HOLMES at ELVIS PRESLEY</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
         <is>
           <t>d13 Tue 21:26</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>MS state line (walk from HOLMES at ELVIS PRESLEY)</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H70" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="I70" t="inlineStr">
         <is>
           <t>walk / local</t>
         </is>
       </c>
-      <c r="J67" t="n">
+      <c r="J70" t="n">
         <v>0.32</v>
       </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr">
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="N67" t="n">
+      <c r="N70" t="n">
         <v>48</v>
       </c>
-      <c r="O67" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
HT 230.02 h, Hanover -> Tallahassee: HMS without its forced Mississippi finish
The 09:00 Memphis -> Birmingham Greyhound stops at Tupelo MS, so HMS's Tallahassee -> Mobile -> Biloxi
finish (forced by --end MS, copied from its sweep run) cost 8.2 h for nothing. 4.2 h under Wheeling,
no Ohio Coach, all 48 verified (Arkansas on the Big River Crossing walk at 05:45, inside the bridge hours).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/route_legs.xlsx
+++ b/docs/route_legs.xlsx
@@ -15,6 +15,7 @@
     <sheet name="X 238.11" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="HAR 237.69" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="HMS 238.19" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="HT 230.02" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31082,4 +31083,3566 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>HT 230.02: 230.02 h, first bus d1 Thu 06:23, finish d10 Sat 20:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Red: connection under 20 min. Green: wait over 2 h. Blue: hand-entered trip (data/manual). Amber: miss penalty of 20 h or more (a once-daily anchor).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>depart</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>arrive</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>ride h</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>wait before h</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>miss penalty h</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>new states</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>total states</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:00</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ledyard Lot</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:04</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>VT state line (walk from Ledyard Lot)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:04</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>VT state line (walk from Ledyard Lot)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:08</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Ledyard Lot</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="n">
+        <v>2</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:23</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ledyard Lot</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:25</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Parkhurst</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Advance Transit: Pink Route</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:25</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Parkhurst</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:33</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:40</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>d1 Thu 09:30</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Dartmouth Coach: Hanover -&gt; Boston South Station 06:40</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>tight, manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>d1 Thu 09:30</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>d1 Thu 09:30</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>d1 Thu 10:00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>d1 Thu 11:55</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>4</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>d1 Thu 12:30</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>d1 Thu 14:25</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>4</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>d1 Thu 14:25</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>d1 Thu 14:33</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="n">
+        <v>4</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>d1 Thu 15:10</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>d1 Thu 21:44</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Baltimore Penn Station</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Amtrak: Acela</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>CT DE MD NJ NY PA RI</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>11</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>d1 Thu 21:44</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Baltimore Penn Station</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>d1 Thu 22:30</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Baltimore Downtown Bus Station</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>11</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>d1 Thu 23:25</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Baltimore Downtown Bus Station</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>d2 Fri 11:25</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Augusta</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>FlixBus-us: NYC Chinatown - Atlanta</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>12</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>GA NC VA</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>14</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>d2 Fri 12:05</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Augusta</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>d2 Fri 13:55</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Camden (McDonald's)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Atlanta - Columbia - Raleigh (Subsidy)</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>15</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>d2 Fri 15:15</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Camden (McDonald's)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>d2 Fri 16:55</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Charlotte Bus Station</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Raleigh - Jacksonville</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>15</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>d2 Fri 16:55</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Charlotte Bus Station</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>d2 Fri 16:55</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>15</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>d2 Fri 17:45</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>d3 Sat 04:30</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Columbus (E Mound St)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Barons Bus Lines: Charlotte -&gt; Columbus</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>KY OH WV</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>18</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>d3 Sat 06:15</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Columbus (E Mound St)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>d3 Sat 12:20</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Michigan City</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Barons Bus Lines: Columbus (E Mound St) -&gt; Chicago</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>19</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>d3 Sat 12:20</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Michigan City</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>d3 Sat 12:21</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Marquette Mall Transfer Point</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>19</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>d3 Sat 12:38</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Marquette Mall Transfer Point</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>d3 Sat 13:09</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Als Karwick</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Michian City Transit: Franklin St./Washington Park/Lakeland/Karwick</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="K22" s="5" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>19</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>d3 Sat 13:09</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Als Karwick</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>d3 Sat 15:00</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Michigan line at Michiana (on foot from Michigan City Carroll Ave)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>20</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>d3 Sat 15:00</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Michigan line at Michiana (on foot from Michigan City Carroll Ave)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>d3 Sat 15:25</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Carroll Ave. (Michigan City)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>20</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>d3 Sat 15:55</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Carroll Ave. (Michigan City)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>d3 Sat 17:19</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Museum Campus/11th St.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Northern Indiana Commuter Transportation District: Lakeshore Corridor</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>21</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>d3 Sat 17:19</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Museum Campus/11th St.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>d3 Sat 17:56</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="n">
+        <v>21</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>d3 Sat 22:00</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>d4 Sun 06:20</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Minneapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Chicago - Milwaukee - Minneapolis</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="K27" s="6" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="L27" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>MN WI</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>23</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>long wait</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>d4 Sun 06:20</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Minneapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>d4 Sun 06:20</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Minneapolis</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="n">
+        <v>23</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>d4 Sun 10:35</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Minneapolis</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>d4 Sun 14:55</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="K29" s="6" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="L29" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>24</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>long wait, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>d4 Sun 15:50</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>d4 Sun 19:50</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Fargo -&gt; Sioux Falls</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>4</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
+        <v>25</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>d4 Sun 20:05</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>d5 Mon 02:15</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Maryville</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Sioux Falls -&gt; Kansas City</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L31" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>IA MO NE</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>28</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>tight, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>d5 Mon 03:25</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Maryville</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>d5 Mon 10:05</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Kansas City -&gt; Sioux Falls</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="K32" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="n">
+        <v>28</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>d5 Mon 12:40</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>d6 Tue 00:25</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="K33" s="6" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="L33" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>MT WY</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>30</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>long wait, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>d6 Tue 01:30</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>d6 Tue 10:30</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Billings -&gt; Spokane</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>10</v>
+      </c>
+      <c r="K34" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="L34" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>ID WA</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>32</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>d6 Tue 10:30</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>d6 Tue 10:30</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="n">
+        <v>32</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>d6 Tue 10:45</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>d6 Tue 13:10</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Northwestern Stage Lines: NWL 710 Spokane -&gt; Pasco</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="K36" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="n">
+        <v>32</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>tight, manual, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>d6 Tue 13:25</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>d7 Wed 02:30</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Salt Lake City Intermodal Trans Ctr</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Seattle-Boise-SLC-Denver</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L37" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>OR UT</t>
+        </is>
+      </c>
+      <c r="N37" t="n">
+        <v>34</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>tight, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>d7 Wed 02:30</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Salt Lake City Intermodal Trans Ctr</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>d7 Wed 03:27</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="n">
+        <v>34</v>
+      </c>
+      <c r="O38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>d7 Wed 04:45</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>d7 Wed 10:20</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Salt Lake Express: SLE 7021 Salt Lake City (Airport) 04:45 -&gt; Saint George (Bluff St Office) 10:20</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="K39" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L39" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="n">
+        <v>34</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>d7 Wed 10:30</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>d7 Wed 11:40</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Las Vegas (Airport)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Salt Lake Express: SLE 8035 Saint George (Bluff St Office) 10:30 -&gt; Las Vegas (Airport) 11:40</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="K40" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>AZ NV</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>36</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>tight, manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>d7 Wed 11:40</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Las Vegas (Airport)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>d7 Wed 12:26</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="n">
+        <v>36</v>
+      </c>
+      <c r="O41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>d7 Wed 14:00</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>d7 Wed 18:15</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>San Bernardino Depot</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Los Angeles - Las Vegas</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="L42" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>37</v>
+      </c>
+      <c r="O42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>d7 Wed 18:15</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>San Bernardino Depot</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>d7 Wed 18:16</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="n">
+        <v>37</v>
+      </c>
+      <c r="O43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>d7 Wed 18:43</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>d9 Fri 01:47</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Amtrak: Southwest Chief</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>29.07</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="L44" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>CO KS NM</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>40</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>d9 Fri 01:47</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>d9 Fri 01:47</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Newton (Amtrak)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="n">
+        <v>40</v>
+      </c>
+      <c r="O45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>d9 Fri 03:00</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Newton (Amtrak)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>d9 Fri 06:38</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Oklahoma (Amtrak)</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Oklahoma City</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="L46" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>41</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>d9 Fri 06:38</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Oklahoma (Amtrak)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>d9 Fri 06:38</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="n">
+        <v>41</v>
+      </c>
+      <c r="O47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>d9 Fri 08:25</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>d9 Fri 12:27</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Amtrak: Heartland Flyer</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="L48" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>42</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>d9 Fri 14:23</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>d9 Fri 18:18</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Longview</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Amtrak: Texas Eagle</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="L49" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="n">
+        <v>42</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>d9 Fri 18:30</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Longview</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>d9 Fri 19:50</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Shreveport Sportran Intermodal Terminal</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Amtrak Chartered Vehicle: Amtrak Thruway Connecting Service</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="K50" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L50" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>43</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>d9 Fri 19:50</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Shreveport Sportran Intermodal Terminal</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>d9 Fri 19:50</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Shreveport Bus Station</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="n">
+        <v>43</v>
+      </c>
+      <c r="O51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>d9 Fri 20:50</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Shreveport Bus Station</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>d9 Fri 22:10</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Texarkana (Travel Stop)</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Texarkana - Houston</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="K52" t="n">
+        <v>1</v>
+      </c>
+      <c r="L52" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="n">
+        <v>43</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>d9 Fri 22:40</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Texarkana (Travel Stop)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>d10 Sat 03:45</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Memphis Bus Station</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Dallas - Nashville - Detroit</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L53" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>44</v>
+      </c>
+      <c r="O53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>d10 Sat 03:45</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Memphis Bus Station</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>d10 Sat 04:54</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="n">
+        <v>44</v>
+      </c>
+      <c r="O54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>d10 Sat 05:45</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>d10 Sat 06:18</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>On foot (Big River Crossing, open 06:00-22:00): Memphis Amtrak -&gt; Arkansas line on Big River Crossing (walk)</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="N55" t="n">
+        <v>45</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>d10 Sat 06:30</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>d10 Sat 07:03</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>On foot (Big River Crossing, open 06:00-22:00): Arkansas line on Big River Crossing -&gt; Memphis Amtrak (walk)</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K56" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L56" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="n">
+        <v>45</v>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>tight, manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>d10 Sat 07:03</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>d10 Sat 08:12</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Memphis Bus Station</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="n">
+        <v>45</v>
+      </c>
+      <c r="O57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>d10 Sat 09:00</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Memphis Bus Station</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>d10 Sat 13:25</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Birmingham Intermodal Facility</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Atlanta - Memphis</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="L58" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>AL MS</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>47</v>
+      </c>
+      <c r="O58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>d10 Sat 13:50</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Birmingham Intermodal Facility</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>d10 Sat 20:25</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Nashville - Tallahassee</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L59" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="N59" t="n">
+        <v>48</v>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
NBA 237.52 h (New Buffalo MI -> Arkansas line); sweep 3 write-up; deferred review fixes
Sweep 3 run 22 focused with the fixed search from its real start stop: 240.5 -> 237.52, verified
independently (all 48), no Ohio Coach. sweep.sh: cd || exit 1, explicit taskkill/kill branch;
time_router: note that rollover offsets assume no DST change in the window. regress 14/14.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/route_legs.xlsx
+++ b/docs/route_legs.xlsx
@@ -16,6 +16,7 @@
     <sheet name="HAR 237.69" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="HMS 238.19" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="HT 230.02" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="NBA 237.52" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4637,6 +4638,3691 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>NBA 237.52: 237.52 h, first bus d7 Wed 21:47, finish d17 Sat 18:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Red: connection under 20 min. Green: wait over 2 h. Blue: hand-entered trip (data/manual). Amber: miss penalty of 20 h or more (a once-daily anchor).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>depart</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>arrive</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>ride h</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>wait before h</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>miss penalty h</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>new states</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>total states</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>d7 Wed 21:47</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>New Buffalo Amtrak</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>d7 Wed 22:25</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Chicago Union Station</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Amtrak: Wolverine</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>IL IN</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>d7 Wed 22:25</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Chicago Union Station</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>d7 Wed 22:37</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>d8 Thu 00:30</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>d8 Thu 08:45</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Saint Paul Union Depot</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Chicago - Milwaukee - Minneapolis</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="L6" t="n">
+        <v>9</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>MN WI</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>d8 Thu 08:45</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Saint Paul Union Depot</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>d8 Thu 08:45</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>St. Paul (Union Depot)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="n">
+        <v>5</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>d8 Thu 09:00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>St. Paul (Union Depot)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>d8 Thu 09:25</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Minneapolis</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Kansas City -&gt; Minneapolis</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>d8 Thu 10:35</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Minneapolis</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>d8 Thu 14:55</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>6</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>d8 Thu 15:50</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>d8 Thu 19:50</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Fargo -&gt; Sioux Falls</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>7</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>d8 Thu 20:05</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>d9 Fri 02:15</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Maryville</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Sioux Falls -&gt; Kansas City</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>IA MO NE</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>10</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>tight, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>d9 Fri 03:25</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Maryville</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>d9 Fri 10:05</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Kansas City -&gt; Sioux Falls</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="n">
+        <v>10</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>d9 Fri 12:40</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>d10 Sat 00:25</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>MT WY</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>12</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>long wait, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>d10 Sat 01:30</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>d10 Sat 10:30</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Jefferson Lines: Billings -&gt; Spokane</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>10</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>ID WA</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>14</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>d10 Sat 10:30</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>d10 Sat 10:30</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>14</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>d10 Sat 10:45</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>d10 Sat 13:10</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Northwestern Stage Lines: NWL 710 Spokane -&gt; Pasco</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="K16" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>14</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>tight, manual, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>d10 Sat 13:25</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>d11 Sun 02:30</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Salt Lake City Intermodal Trans Ctr</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Seattle-Boise-SLC-Denver</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>OR UT</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>16</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>tight, daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>d11 Sun 02:30</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Salt Lake City Intermodal Trans Ctr</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>d11 Sun 03:27</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>16</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>d11 Sun 04:45</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>d11 Sun 10:20</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Salt Lake Express: SLE 7021 Salt Lake City (Airport) 04:45 -&gt; Saint George (Bluff St Office) 10:20</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>16</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>d11 Sun 10:30</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>d11 Sun 11:40</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Las Vegas (Airport)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Salt Lake Express: SLE 8035 Saint George (Bluff St Office) 10:30 -&gt; Las Vegas (Airport) 11:40</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>AZ NV</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>18</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>tight, manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>d11 Sun 11:40</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Las Vegas (Airport)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>d11 Sun 12:26</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>18</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>d11 Sun 14:00</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>d11 Sun 18:15</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>San Bernardino Depot</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Los Angeles - Las Vegas</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="K22" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="L22" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>19</v>
+      </c>
+      <c r="O22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>d11 Sun 18:15</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>San Bernardino Depot</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>d11 Sun 18:16</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>19</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>d11 Sun 18:43</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>d13 Tue 01:47</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Amtrak: Southwest Chief</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>29.07</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>CO KS NM</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>22</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>d13 Tue 01:47</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>d13 Tue 01:47</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Newton (Amtrak)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>22</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>d13 Tue 03:00</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Newton (Amtrak)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>d13 Tue 06:43</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Oklahoma City</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>23</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>d13 Tue 06:43</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>d13 Tue 06:43</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Oklahoma City Bus Station</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="n">
+        <v>23</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>d13 Tue 06:43</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Oklahoma City Bus Station</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>d13 Tue 06:43</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Oklahoma City Bus Station</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="n">
+        <v>23</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>d13 Tue 06:55</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Oklahoma City Bus Station</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>d13 Tue 11:10</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Dallas Bus Station</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Dallas - Oklahoma City - Kansas City</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="K29" s="5" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>24</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>d13 Tue 11:30</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Dallas Bus Station</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>d13 Tue 16:20</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Downtown Houston (Gray St.)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>FlixBus-us: Dallas - Houston</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="L30" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="n">
+        <v>24</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>d13 Tue 16:20</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Downtown Houston (Gray St.)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>d13 Tue 16:43</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Central Station Rusk EB</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="n">
+        <v>24</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>d13 Tue 16:50</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Central Station Rusk EB</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>d13 Tue 17:06</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Magnolia Park Transit Center EB</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Metropolitan Transit Authority of Harris County: METRORAIL GREEN LINE</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="n">
+        <v>24</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>d13 Tue 17:06</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Magnolia Park Transit Center EB</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>d13 Tue 17:07</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Houston Bus Station (Greyhound)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="n">
+        <v>24</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>d13 Tue 18:35</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Houston Bus Station (Greyhound)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>d14 Wed 11:00</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Orlando - Houston</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="K34" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="L34" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>AL FL LA</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>27</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>d14 Wed 11:25</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>d14 Wed 14:50</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Jacksonville (Downtown)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Jacksonville - Mobile</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L35" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="n">
+        <v>27</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>d14 Wed 14:50</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Jacksonville (Downtown)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>d14 Wed 14:50</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>JRTC Bay H</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="n">
+        <v>27</v>
+      </c>
+      <c r="O36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>d14 Wed 15:00</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>JRTC Bay H</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>d14 Wed 15:29</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Amtrak Station</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Jacksonville Transportation Authority: Kings Road</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="n">
+        <v>27</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>d14 Wed 15:29</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Amtrak Station</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>d14 Wed 15:37</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Jacksonville</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="n">
+        <v>27</v>
+      </c>
+      <c r="O38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>d14 Wed 16:11</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Jacksonville</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>d15 Thu 06:25</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Amtrak: Silver Meteor</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>14.23</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="L39" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>GA NC SC VA</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>31</v>
+      </c>
+      <c r="O39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>d15 Thu 06:45</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>d15 Thu 13:56</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Amtrak: Acela</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>CT DE MA MD NJ NY PA RI</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>39</v>
+      </c>
+      <c r="O40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>d15 Thu 13:56</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>d15 Thu 14:04</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="n">
+        <v>39</v>
+      </c>
+      <c r="O41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>d15 Thu 14:15</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>d15 Thu 16:10</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="K42" s="5" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1</v>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>40</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>d15 Thu 16:45</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>d15 Thu 18:40</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="L43" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="n">
+        <v>40</v>
+      </c>
+      <c r="O43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>d15 Thu 18:40</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>d15 Thu 18:40</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="n">
+        <v>40</v>
+      </c>
+      <c r="O44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>d15 Thu 19:30</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>d15 Thu 22:00</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Dartmouth Coach: Boston South Station -&gt; Hanover 19:30</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L45" t="n">
+        <v>2</v>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>41</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>d15 Thu 22:00</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>d15 Thu 22:14</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>VT state line (walk from Hanover (Hanover Inn))</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>42</v>
+      </c>
+      <c r="O46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>d15 Thu 22:14</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>VT state line (walk from Hanover (Hanover Inn))</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>d15 Thu 22:28</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="n">
+        <v>42</v>
+      </c>
+      <c r="O47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>d16 Fri 03:00</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>d16 Fri 06:00</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>Dartmouth Coach: Hanover -&gt; Boston South Station 03:00</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>3</v>
+      </c>
+      <c r="K48" s="6" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="L48" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="n">
+        <v>42</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>long wait, manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>d16 Fri 06:00</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>d16 Fri 06:08</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="n">
+        <v>42</v>
+      </c>
+      <c r="O49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>d16 Fri 07:00</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>d16 Fri 12:17</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Philadelphia</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Amtrak: Acela</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="L50" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="n">
+        <v>42</v>
+      </c>
+      <c r="O50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>d16 Fri 12:42</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Philadelphia</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>d16 Fri 14:26</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Harrisburg</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Amtrak: Pennsylvanian</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="n">
+        <v>42</v>
+      </c>
+      <c r="O51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>d16 Fri 14:26</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Harrisburg</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>d16 Fri 14:26</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Harrisburg Bus Station</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="n">
+        <v>42</v>
+      </c>
+      <c r="O52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>d16 Fri 14:50</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Harrisburg Bus Station</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>d17 Sat 04:10</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Indianapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Greyhound-us: New York - Pittsburgh - St. Louis</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="L53" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>OH WV</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>44</v>
+      </c>
+      <c r="O53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>d17 Sat 04:40</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Indianapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>d17 Sat 09:35</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Nashville Bus Station</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Atlanta - Chicago</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L54" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>KY TN</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>46</v>
+      </c>
+      <c r="O54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>d17 Sat 11:30</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Nashville Bus Station</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>d17 Sat 15:00</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Memphis Bus Station</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>FlixBus-us: Dallas - Nashville</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K55" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="L55" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="n">
+        <v>46</v>
+      </c>
+      <c r="O55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>d17 Sat 15:00</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Memphis Bus Station</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>d17 Sat 15:00</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>AIRWAYS TRANSIT CENTER</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="n">
+        <v>46</v>
+      </c>
+      <c r="O56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>d17 Sat 15:15</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>AIRWAYS TRANSIT CENTER</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>d17 Sat 15:34</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>AIRWAYS BOULEVARD at HOLMES ROAD</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>MATA: CROSSTOWN</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="K57" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L57" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="n">
+        <v>46</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>d17 Sat 15:34</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>AIRWAYS BOULEVARD at HOLMES ROAD</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>d17 Sat 15:54</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>MS state line (walk from AIRWAYS BOULEVARD at HOLMES ROAD)</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>47</v>
+      </c>
+      <c r="O58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>d17 Sat 15:54</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>MS state line (walk from AIRWAYS BOULEVARD at HOLMES ROAD)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>d17 Sat 16:13</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>AIRWAYS BOULEVARD at HOLMES ROAD</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="n">
+        <v>47</v>
+      </c>
+      <c r="O59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>d17 Sat 16:19</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>AIRWAYS BOULEVARD at HOLMES ROAD</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>d17 Sat 16:49</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>ELVIS PRESLEY BLVD at SOUTH PARKWAY EAST</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>MATA: CROSSTOWN</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K60" s="5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="n">
+        <v>47</v>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>d17 Sat 16:49</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>ELVIS PRESLEY BLVD at SOUTH PARKWAY EAST</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>d17 Sat 17:36</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>walk / local</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="n">
+        <v>47</v>
+      </c>
+      <c r="O61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>ride</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>d17 Sat 17:45</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>d17 Sat 18:18</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>On foot (Big River Crossing, open 06:00-22:00): Memphis Amtrak -&gt; Arkansas line on Big River Crossing (walk)</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K62" s="5" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
+        <v>48</v>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>tight, manual</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
HT boards the Flix at Washington Union Station off the Acela (same station; Nick), same 230.02 h
route_report / route_sheets order helper now passes '@stop' pins through.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/route_legs.xlsx
+++ b/docs/route_legs.xlsx
@@ -35445,32 +35445,28 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>d1 Thu 21:44</t>
+          <t>d1 Thu 22:22</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Baltimore Penn Station</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>Amtrak: Acela</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>6.57</v>
+        <v>7.2</v>
       </c>
       <c r="K13" t="n">
         <v>0.61</v>
       </c>
       <c r="L13" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -35493,41 +35489,33 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>d1 Thu 21:44</t>
+          <t>d1 Thu 22:22</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Baltimore Penn Station</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>d1 Thu 22:30</t>
+          <t>d1 Thu 22:22</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Baltimore Downtown Bus Station</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>walk / local</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0.78</v>
+        <v>0.02</v>
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
@@ -35548,19 +35536,15 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>d1 Thu 23:25</t>
+          <t>d2 Fri 00:30</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Baltimore Downtown Bus Station</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>d2 Fri 11:25</t>
@@ -35582,10 +35566,10 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>12</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0.91</v>
+        <v>10.92</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>2.12</v>
       </c>
       <c r="L15" s="4" t="n">
         <v>24</v>
@@ -35600,7 +35584,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>daily anchor</t>
+          <t>long wait, daily anchor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HT starts at Foley Park VT: walk 16 min to the Hanover Inn for the 06:40 Dartmouth Coach (Nick)
Latest start 06:19 under the 5-minute rule (06:20 loses the coach and a day). Drops Advance Transit;
230.10 h from the first step (was 230.25), 229.75 from the first bus. Measured walk link from the
Hanover Inn; regress 14/14.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/route_legs.xlsx
+++ b/docs/route_legs.xlsx
@@ -15,7 +15,7 @@
     <sheet name="X 238.11" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="HAR 237.69" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="HMS 238.19" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="HT 230.02" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="HT 230.10" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="NBA 237.52" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
@@ -34777,7 +34777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O59"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -34800,7 +34800,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HT 230.02: 230.02 h, first bus d1 Thu 06:23, finish d10 Sat 20:25</t>
+          <t>HT 230.10: 229.75 h, first bus d1 Thu 06:40, finish d10 Sat 20:25</t>
         </is>
       </c>
     </row>
@@ -34899,51 +34899,47 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>d1 Thu 06:00</t>
+          <t>d1 Thu 06:19</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ledyard Lot</t>
+          <t>Foley Park at the Vermont end of Ledyard Bridge (on foot to the Hanover Inn)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:35</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>NH</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>d1 Thu 06:04</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>VT state line (walk from Ledyard Lot)</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>VT</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>walk / local</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.27</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>VT</t>
-        </is>
-      </c>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O4" t="inlineStr"/>
     </row>
@@ -34953,54 +34949,66 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>d1 Thu 06:04</t>
+          <t>d1 Thu 06:40</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>VT state line (walk from Ledyard Lot)</t>
+          <t>Hanover (Hanover Inn)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>VT</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>d1 Thu 06:08</t>
+          <t>d1 Thu 09:30</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Ledyard Lot</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>walk / local</t>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Dartmouth Coach: Hanover -&gt; Boston South Station 06:40</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+        <v>2.83</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>MA NH</t>
+        </is>
+      </c>
       <c r="N5" t="n">
-        <v>2</v>
-      </c>
-      <c r="O5" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>tight, manual</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -35008,62 +35016,54 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>d1 Thu 06:23</t>
+          <t>d1 Thu 09:30</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Ledyard Lot</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>d1 Thu 06:25</t>
+          <t>d1 Thu 09:30</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Parkhurst</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Advance Transit: Pink Route</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.2</v>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>tight</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -35071,52 +35071,60 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>d1 Thu 06:25</t>
+          <t>d1 Thu 10:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Parkhurst</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>d1 Thu 06:33</t>
+          <t>d1 Thu 11:55</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Hanover (Hanover Inn)</t>
+          <t>Portland, ME</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+        <v>1.92</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
       <c r="N7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O7" t="inlineStr"/>
     </row>
@@ -35131,22 +35139,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>d1 Thu 06:40</t>
+          <t>d1 Thu 12:30</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Hanover (Hanover Inn)</t>
+          <t>Portland, ME</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>d1 Thu 09:30</t>
+          <t>d1 Thu 14:25</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -35159,33 +35167,25 @@
           <t>MA</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>Dartmouth Coach: Hanover -&gt; Boston South Station 06:40</t>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>2.83</v>
-      </c>
-      <c r="K8" s="5" t="n">
-        <v>0.11</v>
+        <v>1.92</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.58</v>
       </c>
       <c r="L8" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>tight, manual</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -35198,7 +35198,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>d1 Thu 09:30</t>
+          <t>d1 Thu 14:25</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -35213,12 +35213,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>d1 Thu 09:30</t>
+          <t>d1 Thu 14:33</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -35232,13 +35232,13 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.01</v>
+        <v>0.14</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" t="inlineStr"/>
     </row>
@@ -35253,12 +35253,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>d1 Thu 10:00</t>
+          <t>d1 Thu 15:10</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -35268,40 +35268,36 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>d1 Thu 11:55</t>
+          <t>d1 Thu 22:22</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
+          <t>Amtrak: Acela</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>1.92</v>
+        <v>7.2</v>
       </c>
       <c r="K10" t="n">
-        <v>0.49</v>
+        <v>0.61</v>
       </c>
       <c r="L10" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>CT DE MD NJ NY PA RI</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="O10" t="inlineStr"/>
     </row>
@@ -35311,56 +35307,44 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>d1 Thu 12:30</t>
+          <t>d1 Thu 22:22</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>d1 Thu 14:25</t>
+          <t>d1 Thu 22:22</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Concord Coach Lines: Portland, ME to/from Boston &amp; Logan Airport</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
+        <v>0.02</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="O11" t="inlineStr"/>
     </row>
@@ -35370,54 +35354,62 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>d1 Thu 14:25</t>
+          <t>d2 Fri 00:30</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>d1 Thu 14:33</t>
+          <t>d2 Fri 11:25</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Augusta</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>FlixBus-us: NYC Chinatown - Atlanta</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+        <v>10.92</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>GA NC VA</t>
+        </is>
+      </c>
       <c r="N12" t="n">
-        <v>4</v>
-      </c>
-      <c r="O12" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>long wait, daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -35430,53 +35422,61 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>d1 Thu 15:10</t>
+          <t>d2 Fri 12:05</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Augusta</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>d1 Thu 22:22</t>
+          <t>d2 Fri 13:55</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+          <t>Camden (McDonald's)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Amtrak: Acela</t>
+          <t>Greyhound-us: Atlanta - Columbia - Raleigh (Subsidy)</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>7.2</v>
+        <v>1.83</v>
       </c>
       <c r="K13" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="L13" t="n">
-        <v>1</v>
+        <v>0.67</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>22.2</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>CT DE MD NJ NY PA RI</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>11</v>
-      </c>
-      <c r="O13" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -35484,46 +35484,62 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>d1 Thu 22:22</t>
+          <t>d2 Fri 15:15</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>Camden (McDonald's)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>d1 Thu 22:22</t>
+          <t>d2 Fri 16:55</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>Charlotte Bus Station</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Greyhound-us: Raleigh - Jacksonville</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+        <v>1.67</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>24</v>
+      </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>11</v>
-      </c>
-      <c r="O14" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -35531,62 +35547,54 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>d2 Fri 00:30</t>
+          <t>d2 Fri 16:55</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>Charlotte Bus Station</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>d2 Fri 11:25</t>
+          <t>d2 Fri 16:55</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Augusta</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>FlixBus-us: NYC Chinatown - Atlanta</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>10.92</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="L15" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>GA NC VA</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
-        <v>14</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>long wait, daily anchor</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -35599,55 +35607,55 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>d2 Fri 12:05</t>
+          <t>d2 Fri 17:45</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Augusta</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>d2 Fri 13:55</t>
+          <t>d3 Sat 04:30</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Camden (McDonald's)</t>
+          <t>Columbus (E Mound St)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Greyhound-us: Atlanta - Columbia - Raleigh (Subsidy)</t>
+          <t>Barons Bus Lines: Charlotte -&gt; Columbus</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>1.83</v>
+        <v>10.75</v>
       </c>
       <c r="K16" t="n">
-        <v>0.67</v>
+        <v>0.83</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>22.2</v>
+        <v>24</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>KY OH WV</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -35666,51 +35674,55 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>d2 Fri 15:15</t>
+          <t>d3 Sat 06:15</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Camden (McDonald's)</t>
+          <t>Columbus (E Mound St)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>d2 Fri 16:55</t>
+          <t>d3 Sat 12:20</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Charlotte Bus Station</t>
+          <t>Michigan City</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Greyhound-us: Raleigh - Jacksonville</t>
+          <t>Barons Bus Lines: Columbus (E Mound St) -&gt; Chicago</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>1.67</v>
+        <v>7.08</v>
       </c>
       <c r="K17" t="n">
-        <v>1.33</v>
+        <v>1.75</v>
       </c>
       <c r="L17" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
       <c r="N17" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -35729,32 +35741,32 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>d2 Fri 16:55</t>
+          <t>d3 Sat 12:20</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Charlotte Bus Station</t>
+          <t>Michigan City</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>d2 Fri 16:55</t>
+          <t>d3 Sat 12:21</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Marquette Mall Transfer Point</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -35763,13 +35775,13 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="O18" t="inlineStr"/>
     </row>
@@ -35784,59 +35796,55 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>d2 Fri 17:45</t>
+          <t>d3 Sat 12:38</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Marquette Mall Transfer Point</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>d3 Sat 04:30</t>
+          <t>d3 Sat 13:09</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Columbus (E Mound St)</t>
+          <t>Als Karwick</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Barons Bus Lines: Charlotte -&gt; Columbus</t>
+          <t>Michian City Transit: Franklin St./Washington Park/Lakeland/Karwick</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>10.75</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="L19" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>KY OH WV</t>
-        </is>
-      </c>
+        <v>0.52</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>daily anchor</t>
+          <t>tight</t>
         </is>
       </c>
     </row>
@@ -35846,66 +35854,58 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>d3 Sat 06:15</t>
+          <t>d3 Sat 13:09</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Columbus (E Mound St)</t>
+          <t>Als Karwick</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>d3 Sat 12:20</t>
+          <t>d3 Sat 15:00</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Michigan City</t>
+          <t>Michigan line at Michiana (on foot from Michigan City Carroll Ave)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MI</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Barons Bus Lines: Columbus (E Mound St) -&gt; Chicago</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="K20" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>24</v>
-      </c>
+        <v>0.85</v>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MI</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>19</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -35918,47 +35918,47 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>d3 Sat 12:20</t>
+          <t>d3 Sat 15:00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Michigan City</t>
+          <t>Michigan line at Michiana (on foot from Michigan City Carroll Ave)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>d3 Sat 15:25</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Carroll Ave. (Michigan City)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>d3 Sat 12:21</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Marquette Mall Transfer Point</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>walk / local</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>0.03</v>
+        <v>1.42</v>
       </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O21" t="inlineStr"/>
     </row>
@@ -35973,12 +35973,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>d3 Sat 12:38</t>
+          <t>d3 Sat 15:55</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Marquette Mall Transfer Point</t>
+          <t>Carroll Ave. (Michigan City)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -35988,42 +35988,42 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>d3 Sat 13:09</t>
+          <t>d3 Sat 17:19</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Als Karwick</t>
+          <t>Museum Campus/11th St.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Michian City Transit: Franklin St./Washington Park/Lakeland/Karwick</t>
+          <t>Northern Indiana Commuter Transportation District: Lakeshore Corridor</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="K22" s="5" t="n">
-        <v>0.27</v>
+        <v>1.4</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.5</v>
       </c>
       <c r="L22" t="n">
-        <v>1</v>
-      </c>
-      <c r="M22" t="inlineStr"/>
+        <v>1.5</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
       <c r="N22" t="n">
-        <v>19</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>tight</t>
-        </is>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -36036,32 +36036,32 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>d3 Sat 13:09</t>
+          <t>d3 Sat 17:19</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Als Karwick</t>
+          <t>Museum Campus/11th St.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>d3 Sat 15:00</t>
+          <t>d3 Sat 17:56</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Michigan line at Michiana (on foot from Michigan City Carroll Ave)</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -36070,17 +36070,13 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>0.85</v>
+        <v>0.63</v>
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>MI</t>
-        </is>
-      </c>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O23" t="inlineStr"/>
     </row>
@@ -36090,54 +36086,66 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>d3 Sat 15:00</t>
+          <t>d3 Sat 22:00</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Michigan line at Michiana (on foot from Michigan City Carroll Ave)</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>d3 Sat 15:25</t>
+          <t>d4 Sun 06:20</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Carroll Ave. (Michigan City)</t>
+          <t>Minneapolis Bus Station</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Greyhound-us: Chicago - Milwaukee - Minneapolis</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
+        <v>8.33</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="L24" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>MN WI</t>
+        </is>
+      </c>
       <c r="N24" t="n">
-        <v>20</v>
-      </c>
-      <c r="O24" t="inlineStr"/>
+        <v>23</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>long wait</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -36145,60 +36153,52 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>d3 Sat 15:55</t>
+          <t>d4 Sun 06:20</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Carroll Ave. (Michigan City)</t>
+          <t>Minneapolis Bus Station</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>d3 Sat 17:19</t>
+          <t>d4 Sun 06:20</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Museum Campus/11th St.</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Northern Indiana Commuter Transportation District: Lakeshore Corridor</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L25" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O25" t="inlineStr"/>
     </row>
@@ -36208,54 +36208,66 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>d3 Sat 17:19</t>
+          <t>d4 Sun 10:35</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Museum Campus/11th St.</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>d3 Sat 17:56</t>
+          <t>d4 Sun 14:55</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
+        <v>4.33</v>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
       <c r="N26" t="n">
-        <v>21</v>
-      </c>
-      <c r="O26" t="inlineStr"/>
+        <v>24</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>long wait, daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -36268,59 +36280,59 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>d3 Sat 22:00</t>
+          <t>d4 Sun 15:50</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>d4 Sun 06:20</t>
+          <t>d4 Sun 19:50</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Minneapolis Bus Station</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Greyhound-us: Chicago - Milwaukee - Minneapolis</t>
+          <t>Jefferson Lines: Fargo -&gt; Sioux Falls</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="K27" s="6" t="n">
-        <v>4.05</v>
-      </c>
-      <c r="L27" t="n">
-        <v>3.1</v>
+        <v>4</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L27" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>MN WI</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="N27" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>long wait</t>
+          <t>daily anchor</t>
         </is>
       </c>
     </row>
@@ -36330,54 +36342,66 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>d4 Sun 06:20</t>
+          <t>d4 Sun 20:05</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Minneapolis Bus Station</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>d4 Sun 06:20</t>
+          <t>d5 Mon 02:15</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Maryville</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Jefferson Lines: Sioux Falls -&gt; Kansas City</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
+        <v>6.17</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>IA MO NE</t>
+        </is>
+      </c>
       <c r="N28" t="n">
-        <v>23</v>
-      </c>
-      <c r="O28" t="inlineStr"/>
+        <v>28</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>tight, daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -36390,59 +36414,55 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>d4 Sun 10:35</t>
+          <t>d5 Mon 03:25</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Maryville</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>d4 Sun 14:55</t>
+          <t>d5 Mon 10:05</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Fargo</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
+          <t>Jefferson Lines: Kansas City -&gt; Sioux Falls</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="K29" s="6" t="n">
-        <v>4.24</v>
+        <v>6.67</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1.17</v>
       </c>
       <c r="L29" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
+      <c r="M29" t="inlineStr"/>
       <c r="N29" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>long wait, daily anchor</t>
+          <t>daily anchor</t>
         </is>
       </c>
     </row>
@@ -36457,59 +36477,59 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>d4 Sun 15:50</t>
+          <t>d5 Mon 12:40</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Fargo</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>d4 Sun 19:50</t>
+          <t>d6 Tue 00:25</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Billings</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Fargo -&gt; Sioux Falls</t>
+          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>4</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0.92</v>
+        <v>12.75</v>
+      </c>
+      <c r="K30" s="6" t="n">
+        <v>2.58</v>
       </c>
       <c r="L30" s="4" t="n">
         <v>24</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MT WY</t>
         </is>
       </c>
       <c r="N30" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>daily anchor</t>
+          <t>long wait, daily anchor</t>
         </is>
       </c>
     </row>
@@ -36524,59 +36544,59 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>d4 Sun 20:05</t>
+          <t>d6 Tue 01:30</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Billings</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>d5 Mon 02:15</t>
+          <t>d6 Tue 10:30</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Maryville</t>
+          <t>Spokane</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Sioux Falls -&gt; Kansas City</t>
+          <t>Jefferson Lines: Billings -&gt; Spokane</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>6.17</v>
-      </c>
-      <c r="K31" s="5" t="n">
-        <v>0.25</v>
+        <v>10</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1.08</v>
       </c>
       <c r="L31" s="4" t="n">
         <v>24</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>IA MO NE</t>
+          <t>ID WA</t>
         </is>
       </c>
       <c r="N31" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>tight, daily anchor</t>
+          <t>daily anchor</t>
         </is>
       </c>
     </row>
@@ -36586,62 +36606,54 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>d5 Mon 03:25</t>
+          <t>d6 Tue 10:30</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Maryville</t>
+          <t>Spokane</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>d5 Mon 10:05</t>
+          <t>d6 Tue 10:30</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Spokane</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Kansas City -&gt; Sioux Falls</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>6.67</v>
-      </c>
-      <c r="K32" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="L32" s="4" t="n">
-        <v>24</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="n">
-        <v>28</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -36654,59 +36666,55 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>d5 Mon 12:40</t>
+          <t>d6 Tue 10:45</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Spokane</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>d6 Tue 00:25</t>
+          <t>d6 Tue 13:10</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Billings</t>
+          <t>Pasco Bus Stop</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>MT</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Jefferson Lines: Minneapolis -&gt; Billings</t>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Northwestern Stage Lines: NWL 710 Spokane -&gt; Pasco</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>12.75</v>
-      </c>
-      <c r="K33" s="6" t="n">
-        <v>2.58</v>
+        <v>2.42</v>
+      </c>
+      <c r="K33" s="5" t="n">
+        <v>0.25</v>
       </c>
       <c r="L33" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>MT WY</t>
-        </is>
-      </c>
+      <c r="M33" t="inlineStr"/>
       <c r="N33" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>long wait, daily anchor</t>
+          <t>tight, manual, daily anchor</t>
         </is>
       </c>
     </row>
@@ -36721,59 +36729,59 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>d6 Tue 01:30</t>
+          <t>d6 Tue 13:25</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Billings</t>
+          <t>Pasco Bus Stop</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>d6 Tue 10:30</t>
+          <t>d7 Wed 02:30</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Spokane</t>
+          <t>Salt Lake City Intermodal Trans Ctr</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>UT</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Jefferson Lines: Billings -&gt; Spokane</t>
+          <t>Greyhound-us: Seattle-Boise-SLC-Denver</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>10</v>
-      </c>
-      <c r="K34" t="n">
-        <v>1.08</v>
+        <v>12.08</v>
+      </c>
+      <c r="K34" s="5" t="n">
+        <v>0.25</v>
       </c>
       <c r="L34" s="4" t="n">
         <v>24</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>ID WA</t>
+          <t>OR UT</t>
         </is>
       </c>
       <c r="N34" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>daily anchor</t>
+          <t>tight, daily anchor</t>
         </is>
       </c>
     </row>
@@ -36788,32 +36796,32 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>d6 Tue 10:30</t>
+          <t>d7 Wed 02:30</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Spokane</t>
+          <t>Salt Lake City Intermodal Trans Ctr</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>UT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>d6 Tue 10:30</t>
+          <t>d7 Wed 03:27</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Spokane</t>
+          <t>Salt Lake City (Airport)</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>UT</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -36822,13 +36830,13 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O35" t="inlineStr"/>
     </row>
@@ -36843,55 +36851,55 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>d6 Tue 10:45</t>
+          <t>d7 Wed 04:45</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Spokane</t>
+          <t>Salt Lake City (Airport)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>UT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>d6 Tue 13:10</t>
+          <t>d7 Wed 10:20</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Saint George (Bluff St Office)</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>UT</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Northwestern Stage Lines: NWL 710 Spokane -&gt; Pasco</t>
+          <t>Salt Lake Express: SLE 7021 Salt Lake City (Airport) 04:45 -&gt; Saint George (Bluff St Office) 10:20</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>2.42</v>
-      </c>
-      <c r="K36" s="5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L36" s="4" t="n">
-        <v>24</v>
+        <v>5.58</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1.2</v>
       </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>tight, manual, daily anchor</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
@@ -36906,59 +36914,59 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>d6 Tue 13:25</t>
+          <t>d7 Wed 10:30</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Saint George (Bluff St Office)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>UT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>d7 Wed 02:30</t>
+          <t>d7 Wed 11:40</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Salt Lake City Intermodal Trans Ctr</t>
+          <t>Las Vegas (Airport)</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>Greyhound-us: Seattle-Boise-SLC-Denver</t>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Salt Lake Express: SLE 8035 Saint George (Bluff St Office) 10:30 -&gt; Las Vegas (Airport) 11:40</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>12.08</v>
+        <v>2.17</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L37" s="4" t="n">
-        <v>24</v>
+        <v>0.17</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1.5</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>OR UT</t>
+          <t>AZ NV</t>
         </is>
       </c>
       <c r="N37" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>tight, daily anchor</t>
+          <t>tight, manual</t>
         </is>
       </c>
     </row>
@@ -36973,32 +36981,32 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>d7 Wed 02:30</t>
+          <t>d7 Wed 11:40</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Salt Lake City Intermodal Trans Ctr</t>
+          <t>Las Vegas (Airport)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>UT</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>d7 Wed 03:27</t>
+          <t>d7 Wed 12:26</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Salt Lake City (Airport)</t>
+          <t>Las Vegas Bus Terminal</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>UT</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -37007,13 +37015,13 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>0.95</v>
+        <v>0.77</v>
       </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O38" t="inlineStr"/>
     </row>
@@ -37028,57 +37036,57 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>d7 Wed 04:45</t>
+          <t>d7 Wed 14:00</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Salt Lake City (Airport)</t>
+          <t>Las Vegas Bus Terminal</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>UT</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>d7 Wed 10:20</t>
+          <t>d7 Wed 18:15</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>San Bernardino Depot</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>Salt Lake Express: SLE 7021 Salt Lake City (Airport) 04:45 -&gt; Saint George (Bluff St Office) 10:20</t>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Los Angeles - Las Vegas</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>5.58</v>
+        <v>4.25</v>
       </c>
       <c r="K39" t="n">
-        <v>1.3</v>
+        <v>1.56</v>
       </c>
       <c r="L39" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="M39" t="inlineStr"/>
+        <v>12.7</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
       <c r="N39" t="n">
-        <v>34</v>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -37086,66 +37094,54 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>d7 Wed 10:30</t>
+          <t>d7 Wed 18:15</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>San Bernardino Depot</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>UT</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>d7 Wed 11:40</t>
+          <t>d7 Wed 18:16</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Las Vegas (Airport)</t>
+          <t>San Bernardino</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>NV</t>
-        </is>
-      </c>
-      <c r="I40" s="3" t="inlineStr">
-        <is>
-          <t>Salt Lake Express: SLE 8035 Saint George (Bluff St Office) 10:30 -&gt; Las Vegas (Airport) 11:40</t>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>2.17</v>
-      </c>
-      <c r="K40" s="5" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="L40" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>AZ NV</t>
-        </is>
-      </c>
+        <v>0.03</v>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" t="n">
-        <v>36</v>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>tight, manual</t>
-        </is>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -37153,54 +37149,66 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>d7 Wed 11:40</t>
+          <t>d7 Wed 18:43</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Las Vegas (Airport)</t>
+          <t>San Bernardino</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>NV</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>d7 Wed 12:26</t>
+          <t>d9 Fri 01:47</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Las Vegas Bus Terminal</t>
+          <t>Newton</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>NV</t>
+          <t>KS</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Amtrak: Southwest Chief</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
+        <v>29.07</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="L41" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>CO KS NM</t>
+        </is>
+      </c>
       <c r="N41" t="n">
-        <v>36</v>
-      </c>
-      <c r="O41" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -37208,60 +37216,52 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>d7 Wed 14:00</t>
+          <t>d9 Fri 01:47</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Las Vegas Bus Terminal</t>
+          <t>Newton</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>NV</t>
+          <t>KS</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>d7 Wed 18:15</t>
+          <t>d9 Fri 01:47</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>San Bernardino Depot</t>
+          <t>Newton (Amtrak)</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>KS</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Greyhound-us: Los Angeles - Las Vegas</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="K42" t="n">
-        <v>1.56</v>
-      </c>
-      <c r="L42" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
       <c r="N42" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="O42" t="inlineStr"/>
     </row>
@@ -37271,54 +37271,66 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>d7 Wed 18:15</t>
+          <t>d9 Fri 03:00</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>San Bernardino Depot</t>
+          <t>Newton (Amtrak)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>KS</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>d7 Wed 18:16</t>
+          <t>d9 Fri 06:38</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>San Bernardino</t>
+          <t>Oklahoma (Amtrak)</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Oklahoma City</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
+        <v>3.63</v>
+      </c>
+      <c r="K43" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="L43" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="N43" t="n">
-        <v>37</v>
-      </c>
-      <c r="O43" t="inlineStr"/>
+        <v>41</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -37326,66 +37338,54 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>d7 Wed 18:43</t>
+          <t>d9 Fri 06:38</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>San Bernardino</t>
+          <t>Oklahoma (Amtrak)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>d9 Fri 01:47</t>
+          <t>d9 Fri 06:38</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Newton</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>KS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Amtrak: Southwest Chief</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>29.07</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="L44" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>CO KS NM</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
       <c r="N44" t="n">
-        <v>40</v>
-      </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -37393,54 +37393,66 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>d9 Fri 01:47</t>
+          <t>d9 Fri 08:25</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Newton</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>KS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>d9 Fri 01:47</t>
+          <t>d9 Fri 12:27</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Newton (Amtrak)</t>
+          <t>Fort Worth</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>KS</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Amtrak: Heartland Flyer</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
+        <v>4.03</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="L45" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
       <c r="N45" t="n">
-        <v>40</v>
-      </c>
-      <c r="O45" t="inlineStr"/>
+        <v>42</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>daily anchor</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -37453,55 +37465,51 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>d9 Fri 03:00</t>
+          <t>d9 Fri 14:23</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Newton (Amtrak)</t>
+          <t>Fort Worth</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>KS</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>d9 Fri 06:38</t>
+          <t>d9 Fri 18:18</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Oklahoma (Amtrak)</t>
+          <t>Longview</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Oklahoma City</t>
+          <t>Amtrak: Texas Eagle</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>3.63</v>
+        <v>3.92</v>
       </c>
       <c r="K46" t="n">
-        <v>1.21</v>
+        <v>1.93</v>
       </c>
       <c r="L46" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="M46" t="inlineStr"/>
       <c r="N46" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -37515,54 +37523,66 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>d9 Fri 06:38</t>
+          <t>d9 Fri 18:30</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Oklahoma (Amtrak)</t>
+          <t>Longview</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>d9 Fri 06:38</t>
+          <t>d9 Fri 19:50</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Shreveport Sportran Intermodal Terminal</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>Amtrak Chartered Vehicle: Amtrak Thruway Connecting Service</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
-      </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
+        <v>1.33</v>
+      </c>
+      <c r="K47" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L47" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
       <c r="N47" t="n">
-        <v>41</v>
-      </c>
-      <c r="O47" t="inlineStr"/>
+        <v>43</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -37570,66 +37590,54 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>d9 Fri 08:25</t>
+          <t>d9 Fri 19:50</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Shreveport Sportran Intermodal Terminal</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>d9 Fri 12:27</t>
+          <t>d9 Fri 19:50</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Fort Worth</t>
+          <t>Shreveport Bus Station</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Amtrak: Heartland Flyer</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>4.03</v>
-      </c>
-      <c r="K48" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="L48" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
       <c r="N48" t="n">
-        <v>42</v>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>daily anchor</t>
-        </is>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -37642,51 +37650,51 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>d9 Fri 14:23</t>
+          <t>d9 Fri 20:50</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Fort Worth</t>
+          <t>Shreveport Bus Station</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>d9 Fri 22:10</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Texarkana (Travel Stop)</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>d9 Fri 18:18</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Longview</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Amtrak: Texas Eagle</t>
+          <t>Greyhound-us: Texarkana - Houston</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>3.92</v>
+        <v>1.33</v>
       </c>
       <c r="K49" t="n">
-        <v>1.93</v>
+        <v>1</v>
       </c>
       <c r="L49" s="4" t="n">
         <v>24</v>
       </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -37705,12 +37713,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>d9 Fri 18:30</t>
+          <t>d9 Fri 22:40</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Longview</t>
+          <t>Texarkana (Travel Stop)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -37720,46 +37728,42 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>d9 Fri 19:50</t>
+          <t>d10 Sat 03:45</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Shreveport Sportran Intermodal Terminal</t>
+          <t>Memphis Bus Station</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Amtrak Chartered Vehicle: Amtrak Thruway Connecting Service</t>
+          <t>Greyhound-us: Dallas - Nashville - Detroit</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="K50" s="5" t="n">
-        <v>0.2</v>
+        <v>5.08</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0.5</v>
       </c>
       <c r="L50" t="n">
-        <v>14.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="N50" t="n">
-        <v>43</v>
-      </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>tight</t>
-        </is>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -37772,32 +37776,32 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>d9 Fri 19:50</t>
+          <t>d10 Sat 03:45</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Shreveport Sportran Intermodal Terminal</t>
+          <t>Memphis Bus Station</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>d9 Fri 19:50</t>
+          <t>d10 Sat 04:54</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Shreveport Bus Station</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -37806,13 +37810,13 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>1.16</v>
       </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="O51" t="inlineStr"/>
     </row>
@@ -37827,55 +37831,59 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>d9 Fri 20:50</t>
+          <t>d10 Sat 05:45</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Shreveport Bus Station</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>d9 Fri 22:10</t>
+          <t>d10 Sat 06:18</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Texarkana (Travel Stop)</t>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>Greyhound-us: Texarkana - Houston</t>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>On foot (Big River Crossing, open 06:00-22:00): Memphis Amtrak -&gt; Arkansas line on Big River Crossing (walk)</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>1.33</v>
+        <v>0.55</v>
       </c>
       <c r="K52" t="n">
-        <v>1</v>
-      </c>
-      <c r="L52" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M52" t="inlineStr"/>
+        <v>0.84</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
       <c r="N52" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>daily anchor</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
@@ -37890,27 +37898,27 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>d9 Fri 22:40</t>
+          <t>d10 Sat 06:30</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Texarkana (Travel Stop)</t>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>d10 Sat 03:45</t>
+          <t>d10 Sat 07:03</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Memphis Bus Station</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -37918,29 +37926,29 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Greyhound-us: Dallas - Nashville - Detroit</t>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>On foot (Big River Crossing, open 06:00-22:00): Arkansas line on Big River Crossing -&gt; Memphis Amtrak (walk)</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>5.08</v>
-      </c>
-      <c r="K53" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
+      </c>
+      <c r="K53" s="5" t="n">
+        <v>0.2</v>
       </c>
       <c r="L53" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>TN</t>
-        </is>
-      </c>
+        <v>0.2</v>
+      </c>
+      <c r="M53" t="inlineStr"/>
       <c r="N53" t="n">
-        <v>44</v>
-      </c>
-      <c r="O53" t="inlineStr"/>
+        <v>45</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>tight, manual</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -37953,27 +37961,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>d10 Sat 03:45</t>
+          <t>d10 Sat 07:03</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>d10 Sat 08:12</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
           <t>Memphis Bus Station</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>TN</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>d10 Sat 04:54</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Memphis</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -37993,7 +38001,7 @@
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="O54" t="inlineStr"/>
     </row>
@@ -38008,12 +38016,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>d10 Sat 05:45</t>
+          <t>d10 Sat 09:00</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Memphis Bus Station</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -38023,46 +38031,42 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>d10 Sat 06:18</t>
+          <t>d10 Sat 13:25</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+          <t>Birmingham Intermodal Facility</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t>On foot (Big River Crossing, open 06:00-22:00): Memphis Amtrak -&gt; Arkansas line on Big River Crossing (walk)</t>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Atlanta - Memphis</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>0.55</v>
+        <v>4.42</v>
       </c>
       <c r="K55" t="n">
-        <v>0.84</v>
+        <v>0.79</v>
       </c>
       <c r="L55" t="n">
-        <v>0.2</v>
+        <v>12.5</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>AL MS</t>
         </is>
       </c>
       <c r="N55" t="n">
-        <v>45</v>
-      </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -38075,238 +38079,57 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>d10 Sat 06:30</t>
+          <t>d10 Sat 13:50</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+          <t>Birmingham Intermodal Facility</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>d10 Sat 07:03</t>
+          <t>d10 Sat 20:25</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>TN</t>
-        </is>
-      </c>
-      <c r="I56" s="3" t="inlineStr">
-        <is>
-          <t>On foot (Big River Crossing, open 06:00-22:00): Arkansas line on Big River Crossing -&gt; Memphis Amtrak (walk)</t>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Greyhound-us: Nashville - Tallahassee</t>
         </is>
       </c>
       <c r="J56" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="K56" s="5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="L56" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M56" t="inlineStr"/>
+        <v>5.58</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L56" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
       <c r="N56" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="O56" t="inlineStr">
-        <is>
-          <t>tight, manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>54</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>walk</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>d10 Sat 07:03</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Memphis</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>TN</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>d10 Sat 08:12</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>Memphis Bus Station</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>TN</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>walk / local</t>
-        </is>
-      </c>
-      <c r="J57" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="n">
-        <v>45</v>
-      </c>
-      <c r="O57" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>55</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>ride</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>d10 Sat 09:00</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Memphis Bus Station</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>TN</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>d10 Sat 13:25</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>Birmingham Intermodal Facility</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>Greyhound-us: Atlanta - Memphis</t>
-        </is>
-      </c>
-      <c r="J58" t="n">
-        <v>4.42</v>
-      </c>
-      <c r="K58" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="L58" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>AL MS</t>
-        </is>
-      </c>
-      <c r="N58" t="n">
-        <v>47</v>
-      </c>
-      <c r="O58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>56</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>ride</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>d10 Sat 13:50</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Birmingham Intermodal Facility</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>d10 Sat 20:25</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>Greyhound-us: Nashville - Tallahassee</t>
-        </is>
-      </c>
-      <c r="J59" t="n">
-        <v>5.58</v>
-      </c>
-      <c r="K59" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="L59" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="N59" t="n">
-        <v>48</v>
-      </c>
-      <c r="O59" t="inlineStr">
         <is>
           <t>daily anchor</t>
         </is>

</xml_diff>

<commit_message>
Full MATA and lake_erie (allowlist kept for big-city systems); HT's Memphis hop on real Saturday MATA
The MATA allowlist (5 of 25 routes) hid route 39, so HT's Big River Crossing -> Airways Greyhound terminal
hop rode on a local-transit proxy. With all of MATA: route 39 07:23 -> route 30 07:55 -> Airways 08:15,
45 min ahead of the 09:00; Nick's two Google backups (08:17, 08:34) noted. lake_erie was excluded
entirely and is now loaded. Removing every allowlist cost 3.7x connections (13M -> 48M, 2.6 GB router,
~200 s load), so the big-city systems keep theirs (Nick's choice).
Routes: X 238.11 -> 238.05, others unchanged; HT 229.75 from the first bus. regress 14/14. Control
replay 30/39, order MATCH; Holmes menu 376k -> 1.37M (rank 13992 -> 18588, already outside), Conway
menu 34k -> 50k.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/route_legs.xlsx
+++ b/docs/route_legs.xlsx
@@ -23490,7 +23490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O70"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -23513,7 +23513,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>X 238.11: 238.11 h, first bus d3 Sat 22:20, finish d13 Tue 21:26</t>
+          <t>X 238.11: 238.05 h, first bus d3 Sat 22:20, finish d13 Tue 21:23</t>
         </is>
       </c>
     </row>
@@ -27444,12 +27444,12 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>d13 Tue 20:26</t>
+          <t>d13 Tue 20:36</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>BROOKS ROAD at COUGHLIN DRIVE</t>
+          <t>BROOKS RD at 3RD ST</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -27463,7 +27463,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>0.11</v>
+        <v>0.27</v>
       </c>
       <c r="K67" s="5" t="n">
         <v>0.12</v>
@@ -27487,17 +27487,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>ride</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>d13 Tue 20:26</t>
+          <t>d13 Tue 20:43</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>BROOKS ROAD at COUGHLIN DRIVE</t>
+          <t>BROOKS RD at 3RD ST</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -27507,12 +27507,12 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>d13 Tue 20:44</t>
+          <t>d13 Tue 21:03</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>ELVIS PRESLEY BLVD at SPRINGBROOK AVENUE</t>
+          <t>HORN LAKE ROAD at HOLMES ROAD</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -27522,19 +27522,27 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>walk / local</t>
+          <t>MATA: SOUTH THIRD</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
+        <v>0.33</v>
+      </c>
+      <c r="K68" s="5" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="L68" t="n">
+        <v>10</v>
+      </c>
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="n">
         <v>47</v>
       </c>
-      <c r="O68" t="inlineStr"/>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>tight</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -27542,17 +27550,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>d13 Tue 20:51</t>
+          <t>d13 Tue 21:03</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>ELVIS PRESLEY BLVD at SPRINGBROOK AVENUE</t>
+          <t>HORN LAKE ROAD at HOLMES ROAD</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -27562,101 +27570,38 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>d13 Tue 21:07</t>
+          <t>d13 Tue 21:23</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>HOLMES at ELVIS PRESLEY</t>
+          <t>MS state line (walk from HORN LAKE ROAD at HOLMES ROAD)</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>MATA: CROSSTOWN</t>
+          <t>walk / local</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="K69" s="5" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="L69" t="n">
-        <v>8</v>
-      </c>
-      <c r="M69" t="inlineStr"/>
+        <v>0.32</v>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
       <c r="N69" t="n">
-        <v>47</v>
-      </c>
-      <c r="O69" t="inlineStr">
-        <is>
-          <t>tight</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="n">
-        <v>67</v>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>walk</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>d13 Tue 21:07</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>HOLMES at ELVIS PRESLEY</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>TN</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>d13 Tue 21:26</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>MS state line (walk from HOLMES at ELVIS PRESLEY)</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>walk / local</t>
-        </is>
-      </c>
-      <c r="J70" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
-      <c r="N70" t="n">
         <v>48</v>
       </c>
-      <c r="O70" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>